<commit_message>
Generate descriptions for imported sessions
</commit_message>
<xml_diff>
--- a/public/session-import-template.xlsx
+++ b/public/session-import-template.xlsx
@@ -362,7 +362,7 @@
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
       <x:c r="A2" s="2" t="str">
-        <x:v>Fill one row per session. Descriptions are required; each import can contain up to 200 sessions.</x:v>
+        <x:v>Fill one row per session. Descriptions are optional and generated when blank; each import can contain up to 200 sessions.</x:v>
       </x:c>
       <x:c r="B2" s="2"/>
       <x:c r="C2" s="2"/>
@@ -376,7 +376,7 @@
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
       <x:c r="A3" s="2" t="str">
-        <x:v>每行填写一场。英文和中文介绍均为必填；每次最多导入 200 场。</x:v>
+        <x:v>每行填写一场。英文和中文介绍可留空，系统会自动生成；每次最多导入 200 场。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -411,10 +411,10 @@
         <x:v>Formats (singles, doubles) / 形式</x:v>
       </x:c>
       <x:c r="H5" s="13" t="str">
-        <x:v>Description (English) / 英文描述</x:v>
+        <x:v>Description (English, optional) / 英文描述（可选）</x:v>
       </x:c>
       <x:c r="I5" s="13" t="str">
-        <x:v>Description (Chinese) / 中文描述</x:v>
+        <x:v>Description (Chinese, optional) / 中文描述（可选）</x:v>
       </x:c>
       <x:c r="J5" s="13" t="str">
         <x:v>Status (published, draft) / 状态</x:v>
@@ -2942,10 +2942,10 @@
     </x:row>
     <x:row r="12" ht="38" customHeight="1">
       <x:c r="A12" s="14" t="str">
-        <x:v>Descriptions / 活动介绍</x:v>
+        <x:v>Descriptions (optional) / 活动介绍（可选）</x:v>
       </x:c>
       <x:c r="B12" s="14" t="str">
-        <x:v>Both English and Chinese descriptions are required; max 2000 characters each. / 英文和中文介绍均必填，每项最多 2000 字符。</x:v>
+        <x:v>Both English and Chinese descriptions are optional; blank cells are generated from the session details. Max 2000 characters each. / 英文和中文介绍均可留空，留空后会根据场次信息自动生成；每项最多 2000 字符。</x:v>
       </x:c>
       <x:c r="C12" s="14" t="str">
         <x:v>Friendly doubles session</x:v>

</xml_diff>

<commit_message>
Allow Excel imports to create venues
</commit_message>
<xml_diff>
--- a/public/session-import-template.xlsx
+++ b/public/session-import-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sessions" sheetId="1" r:id="Refab5d45d4c3461d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R7f6bf8499003493b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sessions" sheetId="1" r:id="R282aa0e53a41420e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R16ba1330b2f3462e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -362,7 +362,7 @@
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
       <x:c r="A2" s="2" t="str">
-        <x:v>Fill one row per session. Descriptions are optional and generated when blank; each import can contain up to 200 sessions.</x:v>
+        <x:v>Fill one row per session. Missing venues are created automatically with a reused photo; the Excel price stays on the session and is used as the peak default price. Upload up to 200 sessions.</x:v>
       </x:c>
       <x:c r="B2" s="2"/>
       <x:c r="C2" s="2"/>
@@ -376,7 +376,7 @@
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
       <x:c r="A3" s="2" t="str">
-        <x:v>每行填写一场。英文和中文介绍可留空，系统会自动生成；每次最多导入 200 场。</x:v>
+        <x:v>每行填写一场。不存在的场地会自动新建并暂时复用已有照片；Excel 价格保留在场次中，并作为忙时默认价格。每次最多导入 200 场。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -2851,14 +2851,14 @@
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
       <x:c r="A2" s="2" t="str">
-        <x:v>Complete the Sessions sheet and upload the .xlsx file in Admin. Blank rows are ignored.</x:v>
+        <x:v>Complete the Sessions sheet and upload the .xlsx file in Admin. Missing venues are created automatically with a reused photo; the Excel price is kept on the session and used as the peak default price. Blank rows are ignored.</x:v>
       </x:c>
       <x:c r="B2" s="2"/>
       <x:c r="C2" s="2"/>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
       <x:c r="A3" s="2" t="str">
-        <x:v>填写 Sessions 工作表后，在管理员后台上传此 .xlsx 文件。空白行会忽略。</x:v>
+        <x:v>填写 Sessions 工作表后，在管理员后台上传此 .xlsx 文件。不存在的场地会自动新建并暂时复用已有照片；Excel 价格保留在场次中，并作为忙时默认价格。空白行会忽略。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -2874,12 +2874,12 @@
         <x:v>Example / 示例</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="38" customHeight="1">
+    <x:row r="6" ht="78" customHeight="1">
       <x:c r="A6" s="14" t="str">
         <x:v>Venue name / 场地名称</x:v>
       </x:c>
       <x:c r="B6" s="14" t="str">
-        <x:v>Use the exact current English or Chinese name shown in Admin. / 使用后台显示的准确场地名称。</x:v>
+        <x:v>Use the current venue name, or enter a new venue name. New venues use London / 伦敦 as the temporary area, reuse an existing venue photo, and are marked “复用照片” in admin notes. / 可填写现有场地名称，也可填写新场地名称。新场地暂用 London / 伦敦，复用已有场地照片，并在后台备注“复用照片”。</x:v>
       </x:c>
       <x:c r="C6" s="14" t="str">
         <x:v>Use a current venue name</x:v>
@@ -2907,12 +2907,12 @@
         <x:v>18:00 / 20:00</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="38" customHeight="1">
+    <x:row r="9" ht="64" customHeight="1">
       <x:c r="A9" s="14" t="str">
         <x:v>Price per person / 每人价格</x:v>
       </x:c>
       <x:c r="B9" s="14" t="str">
-        <x:v>Enter pounds, not pence. Up to two decimal places. / 填写英镑金额，不是便士，最多两位小数。</x:v>
+        <x:v>Enter pounds, not pence. The exact value becomes the session price and the peak default price for a newly created venue. / 填写英镑金额，不是便士。该数值会作为场次价格；新建场地时也会作为忙时默认价格。</x:v>
       </x:c>
       <x:c r="C9" s="14" t="str">
         <x:v>14.00</x:v>
@@ -2962,12 +2962,12 @@
         <x:v>draft</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="38" customHeight="1">
+    <x:row r="14" ht="64" customHeight="1">
       <x:c r="A14" s="14" t="str">
         <x:v>Duplicate sessions / 重复场次</x:v>
       </x:c>
       <x:c r="B14" s="14" t="str">
-        <x:v>The same venue, date, start time and end time cannot already exist or appear twice in one import. / 同一场地、日期、开始和结束时间不能与已有场次或本次文件中的其他场次重复。</x:v>
+        <x:v>The same venue, date, start time and end time cannot already exist or appear twice in one import. Failed rows show their specific reasons. / 同一场地、日期、开始和结束时间不能与已有场次或本次文件中的其他场次重复。导入失败时会显示具体行和原因。</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str"/>
     </x:row>

</xml_diff>

<commit_message>
Allow admins to preset seeking levels for sessions
</commit_message>
<xml_diff>
--- a/public/session-import-template.xlsx
+++ b/public/session-import-template.xlsx
@@ -344,6 +344,7 @@
     <x:col min="8" max="8" width="38" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="38" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="23" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -359,6 +360,7 @@
       <x:c r="H1" s="1"/>
       <x:c r="I1" s="1"/>
       <x:c r="J1" s="1"/>
+      <x:c r="K1" s="14"/>
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
       <x:c r="A2" s="2" t="str">
@@ -373,6 +375,7 @@
       <x:c r="H2" s="2"/>
       <x:c r="I2" s="2"/>
       <x:c r="J2" s="2"/>
+      <x:c r="K2" s="14"/>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
       <x:c r="A3" s="2" t="str">
@@ -387,6 +390,7 @@
       <x:c r="H3" s="2"/>
       <x:c r="I3" s="2"/>
       <x:c r="J3" s="2"/>
+      <x:c r="K3" s="14"/>
     </x:row>
     <x:row r="5" ht="42" customHeight="1">
       <x:c r="A5" s="13" t="str">
@@ -418,6 +422,9 @@
       </x:c>
       <x:c r="J5" s="13" t="str">
         <x:v>Status (published, draft) / 状态</x:v>
+      </x:c>
+      <x:c r="K5" s="13" t="str">
+        <x:v>Seeking levels (1.0, 1.5) / 寻找水平</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="23" customHeight="1">
@@ -431,6 +438,7 @@
       <x:c r="H6" s="14"/>
       <x:c r="I6" s="14"/>
       <x:c r="J6" s="14"/>
+      <x:c r="K6" s="14"/>
     </x:row>
     <x:row r="7" ht="23" customHeight="1">
       <x:c r="A7" s="14"/>
@@ -443,6 +451,7 @@
       <x:c r="H7" s="14"/>
       <x:c r="I7" s="14"/>
       <x:c r="J7" s="14"/>
+      <x:c r="K7" s="14"/>
     </x:row>
     <x:row r="8" ht="23" customHeight="1">
       <x:c r="A8" s="14"/>
@@ -455,6 +464,7 @@
       <x:c r="H8" s="14"/>
       <x:c r="I8" s="14"/>
       <x:c r="J8" s="14"/>
+      <x:c r="K8" s="14"/>
     </x:row>
     <x:row r="9" ht="23" customHeight="1">
       <x:c r="A9" s="14"/>
@@ -467,6 +477,7 @@
       <x:c r="H9" s="14"/>
       <x:c r="I9" s="14"/>
       <x:c r="J9" s="14"/>
+      <x:c r="K9" s="14"/>
     </x:row>
     <x:row r="10" ht="23" customHeight="1">
       <x:c r="A10" s="14"/>
@@ -479,6 +490,7 @@
       <x:c r="H10" s="14"/>
       <x:c r="I10" s="14"/>
       <x:c r="J10" s="14"/>
+      <x:c r="K10" s="14"/>
     </x:row>
     <x:row r="11" ht="23" customHeight="1">
       <x:c r="A11" s="14"/>
@@ -491,6 +503,7 @@
       <x:c r="H11" s="14"/>
       <x:c r="I11" s="14"/>
       <x:c r="J11" s="14"/>
+      <x:c r="K11" s="14"/>
     </x:row>
     <x:row r="12" ht="23" customHeight="1">
       <x:c r="A12" s="14"/>
@@ -503,6 +516,7 @@
       <x:c r="H12" s="14"/>
       <x:c r="I12" s="14"/>
       <x:c r="J12" s="14"/>
+      <x:c r="K12" s="14"/>
     </x:row>
     <x:row r="13" ht="23" customHeight="1">
       <x:c r="A13" s="14"/>
@@ -515,6 +529,7 @@
       <x:c r="H13" s="14"/>
       <x:c r="I13" s="14"/>
       <x:c r="J13" s="14"/>
+      <x:c r="K13" s="14"/>
     </x:row>
     <x:row r="14" ht="23" customHeight="1">
       <x:c r="A14" s="14"/>
@@ -527,6 +542,7 @@
       <x:c r="H14" s="14"/>
       <x:c r="I14" s="14"/>
       <x:c r="J14" s="14"/>
+      <x:c r="K14" s="14"/>
     </x:row>
     <x:row r="15" ht="23" customHeight="1">
       <x:c r="A15" s="14"/>
@@ -539,6 +555,7 @@
       <x:c r="H15" s="14"/>
       <x:c r="I15" s="14"/>
       <x:c r="J15" s="14"/>
+      <x:c r="K15" s="14"/>
     </x:row>
     <x:row r="16" ht="23" customHeight="1">
       <x:c r="A16" s="14"/>
@@ -551,6 +568,7 @@
       <x:c r="H16" s="14"/>
       <x:c r="I16" s="14"/>
       <x:c r="J16" s="14"/>
+      <x:c r="K16" s="14"/>
     </x:row>
     <x:row r="17" ht="23" customHeight="1">
       <x:c r="A17" s="14"/>
@@ -563,6 +581,7 @@
       <x:c r="H17" s="14"/>
       <x:c r="I17" s="14"/>
       <x:c r="J17" s="14"/>
+      <x:c r="K17" s="14"/>
     </x:row>
     <x:row r="18" ht="23" customHeight="1">
       <x:c r="A18" s="14"/>
@@ -575,6 +594,7 @@
       <x:c r="H18" s="14"/>
       <x:c r="I18" s="14"/>
       <x:c r="J18" s="14"/>
+      <x:c r="K18" s="14"/>
     </x:row>
     <x:row r="19" ht="23" customHeight="1">
       <x:c r="A19" s="14"/>
@@ -587,6 +607,7 @@
       <x:c r="H19" s="14"/>
       <x:c r="I19" s="14"/>
       <x:c r="J19" s="14"/>
+      <x:c r="K19" s="14"/>
     </x:row>
     <x:row r="20" ht="23" customHeight="1">
       <x:c r="A20" s="14"/>
@@ -599,6 +620,7 @@
       <x:c r="H20" s="14"/>
       <x:c r="I20" s="14"/>
       <x:c r="J20" s="14"/>
+      <x:c r="K20" s="14"/>
     </x:row>
     <x:row r="21" ht="23" customHeight="1">
       <x:c r="A21" s="14"/>
@@ -611,6 +633,7 @@
       <x:c r="H21" s="14"/>
       <x:c r="I21" s="14"/>
       <x:c r="J21" s="14"/>
+      <x:c r="K21" s="14"/>
     </x:row>
     <x:row r="22" ht="23" customHeight="1">
       <x:c r="A22" s="14"/>
@@ -623,6 +646,7 @@
       <x:c r="H22" s="14"/>
       <x:c r="I22" s="14"/>
       <x:c r="J22" s="14"/>
+      <x:c r="K22" s="14"/>
     </x:row>
     <x:row r="23" ht="23" customHeight="1">
       <x:c r="A23" s="14"/>
@@ -635,6 +659,7 @@
       <x:c r="H23" s="14"/>
       <x:c r="I23" s="14"/>
       <x:c r="J23" s="14"/>
+      <x:c r="K23" s="14"/>
     </x:row>
     <x:row r="24" ht="23" customHeight="1">
       <x:c r="A24" s="14"/>
@@ -647,6 +672,7 @@
       <x:c r="H24" s="14"/>
       <x:c r="I24" s="14"/>
       <x:c r="J24" s="14"/>
+      <x:c r="K24" s="14"/>
     </x:row>
     <x:row r="25" ht="23" customHeight="1">
       <x:c r="A25" s="14"/>
@@ -659,6 +685,7 @@
       <x:c r="H25" s="14"/>
       <x:c r="I25" s="14"/>
       <x:c r="J25" s="14"/>
+      <x:c r="K25" s="14"/>
     </x:row>
     <x:row r="26" ht="23" customHeight="1">
       <x:c r="A26" s="14"/>
@@ -671,6 +698,7 @@
       <x:c r="H26" s="14"/>
       <x:c r="I26" s="14"/>
       <x:c r="J26" s="14"/>
+      <x:c r="K26" s="14"/>
     </x:row>
     <x:row r="27" ht="23" customHeight="1">
       <x:c r="A27" s="14"/>
@@ -683,6 +711,7 @@
       <x:c r="H27" s="14"/>
       <x:c r="I27" s="14"/>
       <x:c r="J27" s="14"/>
+      <x:c r="K27" s="14"/>
     </x:row>
     <x:row r="28" ht="23" customHeight="1">
       <x:c r="A28" s="14"/>
@@ -695,6 +724,7 @@
       <x:c r="H28" s="14"/>
       <x:c r="I28" s="14"/>
       <x:c r="J28" s="14"/>
+      <x:c r="K28" s="14"/>
     </x:row>
     <x:row r="29" ht="23" customHeight="1">
       <x:c r="A29" s="14"/>
@@ -707,6 +737,7 @@
       <x:c r="H29" s="14"/>
       <x:c r="I29" s="14"/>
       <x:c r="J29" s="14"/>
+      <x:c r="K29" s="14"/>
     </x:row>
     <x:row r="30" ht="23" customHeight="1">
       <x:c r="A30" s="14"/>
@@ -719,6 +750,7 @@
       <x:c r="H30" s="14"/>
       <x:c r="I30" s="14"/>
       <x:c r="J30" s="14"/>
+      <x:c r="K30" s="14"/>
     </x:row>
     <x:row r="31" ht="23" customHeight="1">
       <x:c r="A31" s="14"/>
@@ -731,6 +763,7 @@
       <x:c r="H31" s="14"/>
       <x:c r="I31" s="14"/>
       <x:c r="J31" s="14"/>
+      <x:c r="K31" s="14"/>
     </x:row>
     <x:row r="32" ht="23" customHeight="1">
       <x:c r="A32" s="14"/>
@@ -743,6 +776,7 @@
       <x:c r="H32" s="14"/>
       <x:c r="I32" s="14"/>
       <x:c r="J32" s="14"/>
+      <x:c r="K32" s="14"/>
     </x:row>
     <x:row r="33" ht="23" customHeight="1">
       <x:c r="A33" s="14"/>
@@ -755,6 +789,7 @@
       <x:c r="H33" s="14"/>
       <x:c r="I33" s="14"/>
       <x:c r="J33" s="14"/>
+      <x:c r="K33" s="14"/>
     </x:row>
     <x:row r="34" ht="23" customHeight="1">
       <x:c r="A34" s="14"/>
@@ -767,6 +802,7 @@
       <x:c r="H34" s="14"/>
       <x:c r="I34" s="14"/>
       <x:c r="J34" s="14"/>
+      <x:c r="K34" s="14"/>
     </x:row>
     <x:row r="35" ht="23" customHeight="1">
       <x:c r="A35" s="14"/>
@@ -779,6 +815,7 @@
       <x:c r="H35" s="14"/>
       <x:c r="I35" s="14"/>
       <x:c r="J35" s="14"/>
+      <x:c r="K35" s="14"/>
     </x:row>
     <x:row r="36" ht="23" customHeight="1">
       <x:c r="A36" s="14"/>
@@ -791,6 +828,7 @@
       <x:c r="H36" s="14"/>
       <x:c r="I36" s="14"/>
       <x:c r="J36" s="14"/>
+      <x:c r="K36" s="14"/>
     </x:row>
     <x:row r="37" ht="23" customHeight="1">
       <x:c r="A37" s="14"/>
@@ -803,6 +841,7 @@
       <x:c r="H37" s="14"/>
       <x:c r="I37" s="14"/>
       <x:c r="J37" s="14"/>
+      <x:c r="K37" s="14"/>
     </x:row>
     <x:row r="38" ht="23" customHeight="1">
       <x:c r="A38" s="14"/>
@@ -815,6 +854,7 @@
       <x:c r="H38" s="14"/>
       <x:c r="I38" s="14"/>
       <x:c r="J38" s="14"/>
+      <x:c r="K38" s="14"/>
     </x:row>
     <x:row r="39" ht="23" customHeight="1">
       <x:c r="A39" s="14"/>
@@ -827,6 +867,7 @@
       <x:c r="H39" s="14"/>
       <x:c r="I39" s="14"/>
       <x:c r="J39" s="14"/>
+      <x:c r="K39" s="14"/>
     </x:row>
     <x:row r="40" ht="23" customHeight="1">
       <x:c r="A40" s="14"/>
@@ -839,6 +880,7 @@
       <x:c r="H40" s="14"/>
       <x:c r="I40" s="14"/>
       <x:c r="J40" s="14"/>
+      <x:c r="K40" s="14"/>
     </x:row>
     <x:row r="41" ht="23" customHeight="1">
       <x:c r="A41" s="14"/>
@@ -851,6 +893,7 @@
       <x:c r="H41" s="14"/>
       <x:c r="I41" s="14"/>
       <x:c r="J41" s="14"/>
+      <x:c r="K41" s="14"/>
     </x:row>
     <x:row r="42" ht="23" customHeight="1">
       <x:c r="A42" s="14"/>
@@ -863,6 +906,7 @@
       <x:c r="H42" s="14"/>
       <x:c r="I42" s="14"/>
       <x:c r="J42" s="14"/>
+      <x:c r="K42" s="14"/>
     </x:row>
     <x:row r="43" ht="23" customHeight="1">
       <x:c r="A43" s="14"/>
@@ -875,6 +919,7 @@
       <x:c r="H43" s="14"/>
       <x:c r="I43" s="14"/>
       <x:c r="J43" s="14"/>
+      <x:c r="K43" s="14"/>
     </x:row>
     <x:row r="44" ht="23" customHeight="1">
       <x:c r="A44" s="14"/>
@@ -887,6 +932,7 @@
       <x:c r="H44" s="14"/>
       <x:c r="I44" s="14"/>
       <x:c r="J44" s="14"/>
+      <x:c r="K44" s="14"/>
     </x:row>
     <x:row r="45" ht="23" customHeight="1">
       <x:c r="A45" s="14"/>
@@ -899,6 +945,7 @@
       <x:c r="H45" s="14"/>
       <x:c r="I45" s="14"/>
       <x:c r="J45" s="14"/>
+      <x:c r="K45" s="14"/>
     </x:row>
     <x:row r="46" ht="23" customHeight="1">
       <x:c r="A46" s="14"/>
@@ -911,6 +958,7 @@
       <x:c r="H46" s="14"/>
       <x:c r="I46" s="14"/>
       <x:c r="J46" s="14"/>
+      <x:c r="K46" s="14"/>
     </x:row>
     <x:row r="47" ht="23" customHeight="1">
       <x:c r="A47" s="14"/>
@@ -923,6 +971,7 @@
       <x:c r="H47" s="14"/>
       <x:c r="I47" s="14"/>
       <x:c r="J47" s="14"/>
+      <x:c r="K47" s="14"/>
     </x:row>
     <x:row r="48" ht="23" customHeight="1">
       <x:c r="A48" s="14"/>
@@ -935,6 +984,7 @@
       <x:c r="H48" s="14"/>
       <x:c r="I48" s="14"/>
       <x:c r="J48" s="14"/>
+      <x:c r="K48" s="14"/>
     </x:row>
     <x:row r="49" ht="23" customHeight="1">
       <x:c r="A49" s="14"/>
@@ -947,6 +997,7 @@
       <x:c r="H49" s="14"/>
       <x:c r="I49" s="14"/>
       <x:c r="J49" s="14"/>
+      <x:c r="K49" s="14"/>
     </x:row>
     <x:row r="50" ht="23" customHeight="1">
       <x:c r="A50" s="14"/>
@@ -959,6 +1010,7 @@
       <x:c r="H50" s="14"/>
       <x:c r="I50" s="14"/>
       <x:c r="J50" s="14"/>
+      <x:c r="K50" s="14"/>
     </x:row>
     <x:row r="51" ht="23" customHeight="1">
       <x:c r="A51" s="14"/>
@@ -971,6 +1023,7 @@
       <x:c r="H51" s="14"/>
       <x:c r="I51" s="14"/>
       <x:c r="J51" s="14"/>
+      <x:c r="K51" s="14"/>
     </x:row>
     <x:row r="52" ht="23" customHeight="1">
       <x:c r="A52" s="14"/>
@@ -983,6 +1036,7 @@
       <x:c r="H52" s="14"/>
       <x:c r="I52" s="14"/>
       <x:c r="J52" s="14"/>
+      <x:c r="K52" s="14"/>
     </x:row>
     <x:row r="53" ht="23" customHeight="1">
       <x:c r="A53" s="14"/>
@@ -995,6 +1049,7 @@
       <x:c r="H53" s="14"/>
       <x:c r="I53" s="14"/>
       <x:c r="J53" s="14"/>
+      <x:c r="K53" s="14"/>
     </x:row>
     <x:row r="54" ht="23" customHeight="1">
       <x:c r="A54" s="14"/>
@@ -1007,6 +1062,7 @@
       <x:c r="H54" s="14"/>
       <x:c r="I54" s="14"/>
       <x:c r="J54" s="14"/>
+      <x:c r="K54" s="14"/>
     </x:row>
     <x:row r="55" ht="23" customHeight="1">
       <x:c r="A55" s="14"/>
@@ -1019,6 +1075,7 @@
       <x:c r="H55" s="14"/>
       <x:c r="I55" s="14"/>
       <x:c r="J55" s="14"/>
+      <x:c r="K55" s="14"/>
     </x:row>
     <x:row r="56" ht="23" customHeight="1">
       <x:c r="A56" s="14"/>
@@ -1031,6 +1088,7 @@
       <x:c r="H56" s="14"/>
       <x:c r="I56" s="14"/>
       <x:c r="J56" s="14"/>
+      <x:c r="K56" s="14"/>
     </x:row>
     <x:row r="57" ht="23" customHeight="1">
       <x:c r="A57" s="14"/>
@@ -1043,6 +1101,7 @@
       <x:c r="H57" s="14"/>
       <x:c r="I57" s="14"/>
       <x:c r="J57" s="14"/>
+      <x:c r="K57" s="14"/>
     </x:row>
     <x:row r="58" ht="23" customHeight="1">
       <x:c r="A58" s="14"/>
@@ -1055,6 +1114,7 @@
       <x:c r="H58" s="14"/>
       <x:c r="I58" s="14"/>
       <x:c r="J58" s="14"/>
+      <x:c r="K58" s="14"/>
     </x:row>
     <x:row r="59" ht="23" customHeight="1">
       <x:c r="A59" s="14"/>
@@ -1067,6 +1127,7 @@
       <x:c r="H59" s="14"/>
       <x:c r="I59" s="14"/>
       <x:c r="J59" s="14"/>
+      <x:c r="K59" s="14"/>
     </x:row>
     <x:row r="60" ht="23" customHeight="1">
       <x:c r="A60" s="14"/>
@@ -1079,6 +1140,7 @@
       <x:c r="H60" s="14"/>
       <x:c r="I60" s="14"/>
       <x:c r="J60" s="14"/>
+      <x:c r="K60" s="14"/>
     </x:row>
     <x:row r="61" ht="23" customHeight="1">
       <x:c r="A61" s="14"/>
@@ -1091,6 +1153,7 @@
       <x:c r="H61" s="14"/>
       <x:c r="I61" s="14"/>
       <x:c r="J61" s="14"/>
+      <x:c r="K61" s="14"/>
     </x:row>
     <x:row r="62" ht="23" customHeight="1">
       <x:c r="A62" s="14"/>
@@ -1103,6 +1166,7 @@
       <x:c r="H62" s="14"/>
       <x:c r="I62" s="14"/>
       <x:c r="J62" s="14"/>
+      <x:c r="K62" s="14"/>
     </x:row>
     <x:row r="63" ht="23" customHeight="1">
       <x:c r="A63" s="14"/>
@@ -1115,6 +1179,7 @@
       <x:c r="H63" s="14"/>
       <x:c r="I63" s="14"/>
       <x:c r="J63" s="14"/>
+      <x:c r="K63" s="14"/>
     </x:row>
     <x:row r="64" ht="23" customHeight="1">
       <x:c r="A64" s="14"/>
@@ -1127,6 +1192,7 @@
       <x:c r="H64" s="14"/>
       <x:c r="I64" s="14"/>
       <x:c r="J64" s="14"/>
+      <x:c r="K64" s="14"/>
     </x:row>
     <x:row r="65" ht="23" customHeight="1">
       <x:c r="A65" s="14"/>
@@ -1139,6 +1205,7 @@
       <x:c r="H65" s="14"/>
       <x:c r="I65" s="14"/>
       <x:c r="J65" s="14"/>
+      <x:c r="K65" s="14"/>
     </x:row>
     <x:row r="66" ht="23" customHeight="1">
       <x:c r="A66" s="14"/>
@@ -1151,6 +1218,7 @@
       <x:c r="H66" s="14"/>
       <x:c r="I66" s="14"/>
       <x:c r="J66" s="14"/>
+      <x:c r="K66" s="14"/>
     </x:row>
     <x:row r="67" ht="23" customHeight="1">
       <x:c r="A67" s="14"/>
@@ -1163,6 +1231,7 @@
       <x:c r="H67" s="14"/>
       <x:c r="I67" s="14"/>
       <x:c r="J67" s="14"/>
+      <x:c r="K67" s="14"/>
     </x:row>
     <x:row r="68" ht="23" customHeight="1">
       <x:c r="A68" s="14"/>
@@ -1175,6 +1244,7 @@
       <x:c r="H68" s="14"/>
       <x:c r="I68" s="14"/>
       <x:c r="J68" s="14"/>
+      <x:c r="K68" s="14"/>
     </x:row>
     <x:row r="69" ht="23" customHeight="1">
       <x:c r="A69" s="14"/>
@@ -1187,6 +1257,7 @@
       <x:c r="H69" s="14"/>
       <x:c r="I69" s="14"/>
       <x:c r="J69" s="14"/>
+      <x:c r="K69" s="14"/>
     </x:row>
     <x:row r="70" ht="23" customHeight="1">
       <x:c r="A70" s="14"/>
@@ -1199,6 +1270,7 @@
       <x:c r="H70" s="14"/>
       <x:c r="I70" s="14"/>
       <x:c r="J70" s="14"/>
+      <x:c r="K70" s="14"/>
     </x:row>
     <x:row r="71" ht="23" customHeight="1">
       <x:c r="A71" s="14"/>
@@ -1211,6 +1283,7 @@
       <x:c r="H71" s="14"/>
       <x:c r="I71" s="14"/>
       <x:c r="J71" s="14"/>
+      <x:c r="K71" s="14"/>
     </x:row>
     <x:row r="72" ht="23" customHeight="1">
       <x:c r="A72" s="14"/>
@@ -1223,6 +1296,7 @@
       <x:c r="H72" s="14"/>
       <x:c r="I72" s="14"/>
       <x:c r="J72" s="14"/>
+      <x:c r="K72" s="14"/>
     </x:row>
     <x:row r="73" ht="23" customHeight="1">
       <x:c r="A73" s="14"/>
@@ -1235,6 +1309,7 @@
       <x:c r="H73" s="14"/>
       <x:c r="I73" s="14"/>
       <x:c r="J73" s="14"/>
+      <x:c r="K73" s="14"/>
     </x:row>
     <x:row r="74" ht="23" customHeight="1">
       <x:c r="A74" s="14"/>
@@ -1247,6 +1322,7 @@
       <x:c r="H74" s="14"/>
       <x:c r="I74" s="14"/>
       <x:c r="J74" s="14"/>
+      <x:c r="K74" s="14"/>
     </x:row>
     <x:row r="75" ht="23" customHeight="1">
       <x:c r="A75" s="14"/>
@@ -1259,6 +1335,7 @@
       <x:c r="H75" s="14"/>
       <x:c r="I75" s="14"/>
       <x:c r="J75" s="14"/>
+      <x:c r="K75" s="14"/>
     </x:row>
     <x:row r="76" ht="23" customHeight="1">
       <x:c r="A76" s="14"/>
@@ -1271,6 +1348,7 @@
       <x:c r="H76" s="14"/>
       <x:c r="I76" s="14"/>
       <x:c r="J76" s="14"/>
+      <x:c r="K76" s="14"/>
     </x:row>
     <x:row r="77" ht="23" customHeight="1">
       <x:c r="A77" s="14"/>
@@ -1283,6 +1361,7 @@
       <x:c r="H77" s="14"/>
       <x:c r="I77" s="14"/>
       <x:c r="J77" s="14"/>
+      <x:c r="K77" s="14"/>
     </x:row>
     <x:row r="78" ht="23" customHeight="1">
       <x:c r="A78" s="14"/>
@@ -1295,6 +1374,7 @@
       <x:c r="H78" s="14"/>
       <x:c r="I78" s="14"/>
       <x:c r="J78" s="14"/>
+      <x:c r="K78" s="14"/>
     </x:row>
     <x:row r="79" ht="23" customHeight="1">
       <x:c r="A79" s="14"/>
@@ -1307,6 +1387,7 @@
       <x:c r="H79" s="14"/>
       <x:c r="I79" s="14"/>
       <x:c r="J79" s="14"/>
+      <x:c r="K79" s="14"/>
     </x:row>
     <x:row r="80" ht="23" customHeight="1">
       <x:c r="A80" s="14"/>
@@ -1319,6 +1400,7 @@
       <x:c r="H80" s="14"/>
       <x:c r="I80" s="14"/>
       <x:c r="J80" s="14"/>
+      <x:c r="K80" s="14"/>
     </x:row>
     <x:row r="81" ht="23" customHeight="1">
       <x:c r="A81" s="14"/>
@@ -1331,6 +1413,7 @@
       <x:c r="H81" s="14"/>
       <x:c r="I81" s="14"/>
       <x:c r="J81" s="14"/>
+      <x:c r="K81" s="14"/>
     </x:row>
     <x:row r="82" ht="23" customHeight="1">
       <x:c r="A82" s="14"/>
@@ -1343,6 +1426,7 @@
       <x:c r="H82" s="14"/>
       <x:c r="I82" s="14"/>
       <x:c r="J82" s="14"/>
+      <x:c r="K82" s="14"/>
     </x:row>
     <x:row r="83" ht="23" customHeight="1">
       <x:c r="A83" s="14"/>
@@ -1355,6 +1439,7 @@
       <x:c r="H83" s="14"/>
       <x:c r="I83" s="14"/>
       <x:c r="J83" s="14"/>
+      <x:c r="K83" s="14"/>
     </x:row>
     <x:row r="84" ht="23" customHeight="1">
       <x:c r="A84" s="14"/>
@@ -1367,6 +1452,7 @@
       <x:c r="H84" s="14"/>
       <x:c r="I84" s="14"/>
       <x:c r="J84" s="14"/>
+      <x:c r="K84" s="14"/>
     </x:row>
     <x:row r="85" ht="23" customHeight="1">
       <x:c r="A85" s="14"/>
@@ -1379,6 +1465,7 @@
       <x:c r="H85" s="14"/>
       <x:c r="I85" s="14"/>
       <x:c r="J85" s="14"/>
+      <x:c r="K85" s="14"/>
     </x:row>
     <x:row r="86" ht="23" customHeight="1">
       <x:c r="A86" s="14"/>
@@ -1391,6 +1478,7 @@
       <x:c r="H86" s="14"/>
       <x:c r="I86" s="14"/>
       <x:c r="J86" s="14"/>
+      <x:c r="K86" s="14"/>
     </x:row>
     <x:row r="87" ht="23" customHeight="1">
       <x:c r="A87" s="14"/>
@@ -1403,6 +1491,7 @@
       <x:c r="H87" s="14"/>
       <x:c r="I87" s="14"/>
       <x:c r="J87" s="14"/>
+      <x:c r="K87" s="14"/>
     </x:row>
     <x:row r="88" ht="23" customHeight="1">
       <x:c r="A88" s="14"/>
@@ -1415,6 +1504,7 @@
       <x:c r="H88" s="14"/>
       <x:c r="I88" s="14"/>
       <x:c r="J88" s="14"/>
+      <x:c r="K88" s="14"/>
     </x:row>
     <x:row r="89" ht="23" customHeight="1">
       <x:c r="A89" s="14"/>
@@ -1427,6 +1517,7 @@
       <x:c r="H89" s="14"/>
       <x:c r="I89" s="14"/>
       <x:c r="J89" s="14"/>
+      <x:c r="K89" s="14"/>
     </x:row>
     <x:row r="90" ht="23" customHeight="1">
       <x:c r="A90" s="14"/>
@@ -1439,6 +1530,7 @@
       <x:c r="H90" s="14"/>
       <x:c r="I90" s="14"/>
       <x:c r="J90" s="14"/>
+      <x:c r="K90" s="14"/>
     </x:row>
     <x:row r="91" ht="23" customHeight="1">
       <x:c r="A91" s="14"/>
@@ -1451,6 +1543,7 @@
       <x:c r="H91" s="14"/>
       <x:c r="I91" s="14"/>
       <x:c r="J91" s="14"/>
+      <x:c r="K91" s="14"/>
     </x:row>
     <x:row r="92" ht="23" customHeight="1">
       <x:c r="A92" s="14"/>
@@ -1463,6 +1556,7 @@
       <x:c r="H92" s="14"/>
       <x:c r="I92" s="14"/>
       <x:c r="J92" s="14"/>
+      <x:c r="K92" s="14"/>
     </x:row>
     <x:row r="93" ht="23" customHeight="1">
       <x:c r="A93" s="14"/>
@@ -1475,6 +1569,7 @@
       <x:c r="H93" s="14"/>
       <x:c r="I93" s="14"/>
       <x:c r="J93" s="14"/>
+      <x:c r="K93" s="14"/>
     </x:row>
     <x:row r="94" ht="23" customHeight="1">
       <x:c r="A94" s="14"/>
@@ -1487,6 +1582,7 @@
       <x:c r="H94" s="14"/>
       <x:c r="I94" s="14"/>
       <x:c r="J94" s="14"/>
+      <x:c r="K94" s="14"/>
     </x:row>
     <x:row r="95" ht="23" customHeight="1">
       <x:c r="A95" s="14"/>
@@ -1499,6 +1595,7 @@
       <x:c r="H95" s="14"/>
       <x:c r="I95" s="14"/>
       <x:c r="J95" s="14"/>
+      <x:c r="K95" s="14"/>
     </x:row>
     <x:row r="96" ht="23" customHeight="1">
       <x:c r="A96" s="14"/>
@@ -1511,6 +1608,7 @@
       <x:c r="H96" s="14"/>
       <x:c r="I96" s="14"/>
       <x:c r="J96" s="14"/>
+      <x:c r="K96" s="14"/>
     </x:row>
     <x:row r="97" ht="23" customHeight="1">
       <x:c r="A97" s="14"/>
@@ -1523,6 +1621,7 @@
       <x:c r="H97" s="14"/>
       <x:c r="I97" s="14"/>
       <x:c r="J97" s="14"/>
+      <x:c r="K97" s="14"/>
     </x:row>
     <x:row r="98" ht="23" customHeight="1">
       <x:c r="A98" s="14"/>
@@ -1535,6 +1634,7 @@
       <x:c r="H98" s="14"/>
       <x:c r="I98" s="14"/>
       <x:c r="J98" s="14"/>
+      <x:c r="K98" s="14"/>
     </x:row>
     <x:row r="99" ht="23" customHeight="1">
       <x:c r="A99" s="14"/>
@@ -1547,6 +1647,7 @@
       <x:c r="H99" s="14"/>
       <x:c r="I99" s="14"/>
       <x:c r="J99" s="14"/>
+      <x:c r="K99" s="14"/>
     </x:row>
     <x:row r="100" ht="23" customHeight="1">
       <x:c r="A100" s="14"/>
@@ -1559,6 +1660,7 @@
       <x:c r="H100" s="14"/>
       <x:c r="I100" s="14"/>
       <x:c r="J100" s="14"/>
+      <x:c r="K100" s="14"/>
     </x:row>
     <x:row r="101" ht="23" customHeight="1">
       <x:c r="A101" s="14"/>
@@ -1571,6 +1673,7 @@
       <x:c r="H101" s="14"/>
       <x:c r="I101" s="14"/>
       <x:c r="J101" s="14"/>
+      <x:c r="K101" s="14"/>
     </x:row>
     <x:row r="102" ht="23" customHeight="1">
       <x:c r="A102" s="14"/>
@@ -1583,6 +1686,7 @@
       <x:c r="H102" s="14"/>
       <x:c r="I102" s="14"/>
       <x:c r="J102" s="14"/>
+      <x:c r="K102" s="14"/>
     </x:row>
     <x:row r="103" ht="23" customHeight="1">
       <x:c r="A103" s="14"/>
@@ -1595,6 +1699,7 @@
       <x:c r="H103" s="14"/>
       <x:c r="I103" s="14"/>
       <x:c r="J103" s="14"/>
+      <x:c r="K103" s="14"/>
     </x:row>
     <x:row r="104" ht="23" customHeight="1">
       <x:c r="A104" s="14"/>
@@ -1607,6 +1712,7 @@
       <x:c r="H104" s="14"/>
       <x:c r="I104" s="14"/>
       <x:c r="J104" s="14"/>
+      <x:c r="K104" s="14"/>
     </x:row>
     <x:row r="105" ht="23" customHeight="1">
       <x:c r="A105" s="14"/>
@@ -1619,6 +1725,7 @@
       <x:c r="H105" s="14"/>
       <x:c r="I105" s="14"/>
       <x:c r="J105" s="14"/>
+      <x:c r="K105" s="14"/>
     </x:row>
     <x:row r="106" ht="23" customHeight="1">
       <x:c r="A106" s="14"/>
@@ -1631,6 +1738,7 @@
       <x:c r="H106" s="14"/>
       <x:c r="I106" s="14"/>
       <x:c r="J106" s="14"/>
+      <x:c r="K106" s="14"/>
     </x:row>
     <x:row r="107" ht="23" customHeight="1">
       <x:c r="A107" s="14"/>
@@ -1643,6 +1751,7 @@
       <x:c r="H107" s="14"/>
       <x:c r="I107" s="14"/>
       <x:c r="J107" s="14"/>
+      <x:c r="K107" s="14"/>
     </x:row>
     <x:row r="108" ht="23" customHeight="1">
       <x:c r="A108" s="14"/>
@@ -1655,6 +1764,7 @@
       <x:c r="H108" s="14"/>
       <x:c r="I108" s="14"/>
       <x:c r="J108" s="14"/>
+      <x:c r="K108" s="14"/>
     </x:row>
     <x:row r="109" ht="23" customHeight="1">
       <x:c r="A109" s="14"/>
@@ -1667,6 +1777,7 @@
       <x:c r="H109" s="14"/>
       <x:c r="I109" s="14"/>
       <x:c r="J109" s="14"/>
+      <x:c r="K109" s="14"/>
     </x:row>
     <x:row r="110" ht="23" customHeight="1">
       <x:c r="A110" s="14"/>
@@ -1679,6 +1790,7 @@
       <x:c r="H110" s="14"/>
       <x:c r="I110" s="14"/>
       <x:c r="J110" s="14"/>
+      <x:c r="K110" s="14"/>
     </x:row>
     <x:row r="111" ht="23" customHeight="1">
       <x:c r="A111" s="14"/>
@@ -1691,6 +1803,7 @@
       <x:c r="H111" s="14"/>
       <x:c r="I111" s="14"/>
       <x:c r="J111" s="14"/>
+      <x:c r="K111" s="14"/>
     </x:row>
     <x:row r="112" ht="23" customHeight="1">
       <x:c r="A112" s="14"/>
@@ -1703,6 +1816,7 @@
       <x:c r="H112" s="14"/>
       <x:c r="I112" s="14"/>
       <x:c r="J112" s="14"/>
+      <x:c r="K112" s="14"/>
     </x:row>
     <x:row r="113" ht="23" customHeight="1">
       <x:c r="A113" s="14"/>
@@ -1715,6 +1829,7 @@
       <x:c r="H113" s="14"/>
       <x:c r="I113" s="14"/>
       <x:c r="J113" s="14"/>
+      <x:c r="K113" s="14"/>
     </x:row>
     <x:row r="114" ht="23" customHeight="1">
       <x:c r="A114" s="14"/>
@@ -1727,6 +1842,7 @@
       <x:c r="H114" s="14"/>
       <x:c r="I114" s="14"/>
       <x:c r="J114" s="14"/>
+      <x:c r="K114" s="14"/>
     </x:row>
     <x:row r="115" ht="23" customHeight="1">
       <x:c r="A115" s="14"/>
@@ -1739,6 +1855,7 @@
       <x:c r="H115" s="14"/>
       <x:c r="I115" s="14"/>
       <x:c r="J115" s="14"/>
+      <x:c r="K115" s="14"/>
     </x:row>
     <x:row r="116" ht="23" customHeight="1">
       <x:c r="A116" s="14"/>
@@ -1751,6 +1868,7 @@
       <x:c r="H116" s="14"/>
       <x:c r="I116" s="14"/>
       <x:c r="J116" s="14"/>
+      <x:c r="K116" s="14"/>
     </x:row>
     <x:row r="117" ht="23" customHeight="1">
       <x:c r="A117" s="14"/>
@@ -1763,6 +1881,7 @@
       <x:c r="H117" s="14"/>
       <x:c r="I117" s="14"/>
       <x:c r="J117" s="14"/>
+      <x:c r="K117" s="14"/>
     </x:row>
     <x:row r="118" ht="23" customHeight="1">
       <x:c r="A118" s="14"/>
@@ -1775,6 +1894,7 @@
       <x:c r="H118" s="14"/>
       <x:c r="I118" s="14"/>
       <x:c r="J118" s="14"/>
+      <x:c r="K118" s="14"/>
     </x:row>
     <x:row r="119" ht="23" customHeight="1">
       <x:c r="A119" s="14"/>
@@ -1787,6 +1907,7 @@
       <x:c r="H119" s="14"/>
       <x:c r="I119" s="14"/>
       <x:c r="J119" s="14"/>
+      <x:c r="K119" s="14"/>
     </x:row>
     <x:row r="120" ht="23" customHeight="1">
       <x:c r="A120" s="14"/>
@@ -1799,6 +1920,7 @@
       <x:c r="H120" s="14"/>
       <x:c r="I120" s="14"/>
       <x:c r="J120" s="14"/>
+      <x:c r="K120" s="14"/>
     </x:row>
     <x:row r="121" ht="23" customHeight="1">
       <x:c r="A121" s="14"/>
@@ -1811,6 +1933,7 @@
       <x:c r="H121" s="14"/>
       <x:c r="I121" s="14"/>
       <x:c r="J121" s="14"/>
+      <x:c r="K121" s="14"/>
     </x:row>
     <x:row r="122" ht="23" customHeight="1">
       <x:c r="A122" s="14"/>
@@ -1823,6 +1946,7 @@
       <x:c r="H122" s="14"/>
       <x:c r="I122" s="14"/>
       <x:c r="J122" s="14"/>
+      <x:c r="K122" s="14"/>
     </x:row>
     <x:row r="123" ht="23" customHeight="1">
       <x:c r="A123" s="14"/>
@@ -1835,6 +1959,7 @@
       <x:c r="H123" s="14"/>
       <x:c r="I123" s="14"/>
       <x:c r="J123" s="14"/>
+      <x:c r="K123" s="14"/>
     </x:row>
     <x:row r="124" ht="23" customHeight="1">
       <x:c r="A124" s="14"/>
@@ -1847,6 +1972,7 @@
       <x:c r="H124" s="14"/>
       <x:c r="I124" s="14"/>
       <x:c r="J124" s="14"/>
+      <x:c r="K124" s="14"/>
     </x:row>
     <x:row r="125" ht="23" customHeight="1">
       <x:c r="A125" s="14"/>
@@ -1859,6 +1985,7 @@
       <x:c r="H125" s="14"/>
       <x:c r="I125" s="14"/>
       <x:c r="J125" s="14"/>
+      <x:c r="K125" s="14"/>
     </x:row>
     <x:row r="126" ht="23" customHeight="1">
       <x:c r="A126" s="14"/>
@@ -1871,6 +1998,7 @@
       <x:c r="H126" s="14"/>
       <x:c r="I126" s="14"/>
       <x:c r="J126" s="14"/>
+      <x:c r="K126" s="14"/>
     </x:row>
     <x:row r="127" ht="23" customHeight="1">
       <x:c r="A127" s="14"/>
@@ -1883,6 +2011,7 @@
       <x:c r="H127" s="14"/>
       <x:c r="I127" s="14"/>
       <x:c r="J127" s="14"/>
+      <x:c r="K127" s="14"/>
     </x:row>
     <x:row r="128" ht="23" customHeight="1">
       <x:c r="A128" s="14"/>
@@ -1895,6 +2024,7 @@
       <x:c r="H128" s="14"/>
       <x:c r="I128" s="14"/>
       <x:c r="J128" s="14"/>
+      <x:c r="K128" s="14"/>
     </x:row>
     <x:row r="129" ht="23" customHeight="1">
       <x:c r="A129" s="14"/>
@@ -1907,6 +2037,7 @@
       <x:c r="H129" s="14"/>
       <x:c r="I129" s="14"/>
       <x:c r="J129" s="14"/>
+      <x:c r="K129" s="14"/>
     </x:row>
     <x:row r="130" ht="23" customHeight="1">
       <x:c r="A130" s="14"/>
@@ -1919,6 +2050,7 @@
       <x:c r="H130" s="14"/>
       <x:c r="I130" s="14"/>
       <x:c r="J130" s="14"/>
+      <x:c r="K130" s="14"/>
     </x:row>
     <x:row r="131" ht="23" customHeight="1">
       <x:c r="A131" s="14"/>
@@ -1931,6 +2063,7 @@
       <x:c r="H131" s="14"/>
       <x:c r="I131" s="14"/>
       <x:c r="J131" s="14"/>
+      <x:c r="K131" s="14"/>
     </x:row>
     <x:row r="132" ht="23" customHeight="1">
       <x:c r="A132" s="14"/>
@@ -1943,6 +2076,7 @@
       <x:c r="H132" s="14"/>
       <x:c r="I132" s="14"/>
       <x:c r="J132" s="14"/>
+      <x:c r="K132" s="14"/>
     </x:row>
     <x:row r="133" ht="23" customHeight="1">
       <x:c r="A133" s="14"/>
@@ -1955,6 +2089,7 @@
       <x:c r="H133" s="14"/>
       <x:c r="I133" s="14"/>
       <x:c r="J133" s="14"/>
+      <x:c r="K133" s="14"/>
     </x:row>
     <x:row r="134" ht="23" customHeight="1">
       <x:c r="A134" s="14"/>
@@ -1967,6 +2102,7 @@
       <x:c r="H134" s="14"/>
       <x:c r="I134" s="14"/>
       <x:c r="J134" s="14"/>
+      <x:c r="K134" s="14"/>
     </x:row>
     <x:row r="135" ht="23" customHeight="1">
       <x:c r="A135" s="14"/>
@@ -1979,6 +2115,7 @@
       <x:c r="H135" s="14"/>
       <x:c r="I135" s="14"/>
       <x:c r="J135" s="14"/>
+      <x:c r="K135" s="14"/>
     </x:row>
     <x:row r="136" ht="23" customHeight="1">
       <x:c r="A136" s="14"/>
@@ -1991,6 +2128,7 @@
       <x:c r="H136" s="14"/>
       <x:c r="I136" s="14"/>
       <x:c r="J136" s="14"/>
+      <x:c r="K136" s="14"/>
     </x:row>
     <x:row r="137" ht="23" customHeight="1">
       <x:c r="A137" s="14"/>
@@ -2003,6 +2141,7 @@
       <x:c r="H137" s="14"/>
       <x:c r="I137" s="14"/>
       <x:c r="J137" s="14"/>
+      <x:c r="K137" s="14"/>
     </x:row>
     <x:row r="138" ht="23" customHeight="1">
       <x:c r="A138" s="14"/>
@@ -2015,6 +2154,7 @@
       <x:c r="H138" s="14"/>
       <x:c r="I138" s="14"/>
       <x:c r="J138" s="14"/>
+      <x:c r="K138" s="14"/>
     </x:row>
     <x:row r="139" ht="23" customHeight="1">
       <x:c r="A139" s="14"/>
@@ -2027,6 +2167,7 @@
       <x:c r="H139" s="14"/>
       <x:c r="I139" s="14"/>
       <x:c r="J139" s="14"/>
+      <x:c r="K139" s="14"/>
     </x:row>
     <x:row r="140" ht="23" customHeight="1">
       <x:c r="A140" s="14"/>
@@ -2039,6 +2180,7 @@
       <x:c r="H140" s="14"/>
       <x:c r="I140" s="14"/>
       <x:c r="J140" s="14"/>
+      <x:c r="K140" s="14"/>
     </x:row>
     <x:row r="141" ht="23" customHeight="1">
       <x:c r="A141" s="14"/>
@@ -2051,6 +2193,7 @@
       <x:c r="H141" s="14"/>
       <x:c r="I141" s="14"/>
       <x:c r="J141" s="14"/>
+      <x:c r="K141" s="14"/>
     </x:row>
     <x:row r="142" ht="23" customHeight="1">
       <x:c r="A142" s="14"/>
@@ -2063,6 +2206,7 @@
       <x:c r="H142" s="14"/>
       <x:c r="I142" s="14"/>
       <x:c r="J142" s="14"/>
+      <x:c r="K142" s="14"/>
     </x:row>
     <x:row r="143" ht="23" customHeight="1">
       <x:c r="A143" s="14"/>
@@ -2075,6 +2219,7 @@
       <x:c r="H143" s="14"/>
       <x:c r="I143" s="14"/>
       <x:c r="J143" s="14"/>
+      <x:c r="K143" s="14"/>
     </x:row>
     <x:row r="144" ht="23" customHeight="1">
       <x:c r="A144" s="14"/>
@@ -2087,6 +2232,7 @@
       <x:c r="H144" s="14"/>
       <x:c r="I144" s="14"/>
       <x:c r="J144" s="14"/>
+      <x:c r="K144" s="14"/>
     </x:row>
     <x:row r="145" ht="23" customHeight="1">
       <x:c r="A145" s="14"/>
@@ -2099,6 +2245,7 @@
       <x:c r="H145" s="14"/>
       <x:c r="I145" s="14"/>
       <x:c r="J145" s="14"/>
+      <x:c r="K145" s="14"/>
     </x:row>
     <x:row r="146" ht="23" customHeight="1">
       <x:c r="A146" s="14"/>
@@ -2111,6 +2258,7 @@
       <x:c r="H146" s="14"/>
       <x:c r="I146" s="14"/>
       <x:c r="J146" s="14"/>
+      <x:c r="K146" s="14"/>
     </x:row>
     <x:row r="147" ht="23" customHeight="1">
       <x:c r="A147" s="14"/>
@@ -2123,6 +2271,7 @@
       <x:c r="H147" s="14"/>
       <x:c r="I147" s="14"/>
       <x:c r="J147" s="14"/>
+      <x:c r="K147" s="14"/>
     </x:row>
     <x:row r="148" ht="23" customHeight="1">
       <x:c r="A148" s="14"/>
@@ -2135,6 +2284,7 @@
       <x:c r="H148" s="14"/>
       <x:c r="I148" s="14"/>
       <x:c r="J148" s="14"/>
+      <x:c r="K148" s="14"/>
     </x:row>
     <x:row r="149" ht="23" customHeight="1">
       <x:c r="A149" s="14"/>
@@ -2147,6 +2297,7 @@
       <x:c r="H149" s="14"/>
       <x:c r="I149" s="14"/>
       <x:c r="J149" s="14"/>
+      <x:c r="K149" s="14"/>
     </x:row>
     <x:row r="150" ht="23" customHeight="1">
       <x:c r="A150" s="14"/>
@@ -2159,6 +2310,7 @@
       <x:c r="H150" s="14"/>
       <x:c r="I150" s="14"/>
       <x:c r="J150" s="14"/>
+      <x:c r="K150" s="14"/>
     </x:row>
     <x:row r="151" ht="23" customHeight="1">
       <x:c r="A151" s="14"/>
@@ -2171,6 +2323,7 @@
       <x:c r="H151" s="14"/>
       <x:c r="I151" s="14"/>
       <x:c r="J151" s="14"/>
+      <x:c r="K151" s="14"/>
     </x:row>
     <x:row r="152" ht="23" customHeight="1">
       <x:c r="A152" s="14"/>
@@ -2183,6 +2336,7 @@
       <x:c r="H152" s="14"/>
       <x:c r="I152" s="14"/>
       <x:c r="J152" s="14"/>
+      <x:c r="K152" s="14"/>
     </x:row>
     <x:row r="153" ht="23" customHeight="1">
       <x:c r="A153" s="14"/>
@@ -2195,6 +2349,7 @@
       <x:c r="H153" s="14"/>
       <x:c r="I153" s="14"/>
       <x:c r="J153" s="14"/>
+      <x:c r="K153" s="14"/>
     </x:row>
     <x:row r="154" ht="23" customHeight="1">
       <x:c r="A154" s="14"/>
@@ -2207,6 +2362,7 @@
       <x:c r="H154" s="14"/>
       <x:c r="I154" s="14"/>
       <x:c r="J154" s="14"/>
+      <x:c r="K154" s="14"/>
     </x:row>
     <x:row r="155" ht="23" customHeight="1">
       <x:c r="A155" s="14"/>
@@ -2219,6 +2375,7 @@
       <x:c r="H155" s="14"/>
       <x:c r="I155" s="14"/>
       <x:c r="J155" s="14"/>
+      <x:c r="K155" s="14"/>
     </x:row>
     <x:row r="156" ht="23" customHeight="1">
       <x:c r="A156" s="14"/>
@@ -2231,6 +2388,7 @@
       <x:c r="H156" s="14"/>
       <x:c r="I156" s="14"/>
       <x:c r="J156" s="14"/>
+      <x:c r="K156" s="14"/>
     </x:row>
     <x:row r="157" ht="23" customHeight="1">
       <x:c r="A157" s="14"/>
@@ -2243,6 +2401,7 @@
       <x:c r="H157" s="14"/>
       <x:c r="I157" s="14"/>
       <x:c r="J157" s="14"/>
+      <x:c r="K157" s="14"/>
     </x:row>
     <x:row r="158" ht="23" customHeight="1">
       <x:c r="A158" s="14"/>
@@ -2255,6 +2414,7 @@
       <x:c r="H158" s="14"/>
       <x:c r="I158" s="14"/>
       <x:c r="J158" s="14"/>
+      <x:c r="K158" s="14"/>
     </x:row>
     <x:row r="159" ht="23" customHeight="1">
       <x:c r="A159" s="14"/>
@@ -2267,6 +2427,7 @@
       <x:c r="H159" s="14"/>
       <x:c r="I159" s="14"/>
       <x:c r="J159" s="14"/>
+      <x:c r="K159" s="14"/>
     </x:row>
     <x:row r="160" ht="23" customHeight="1">
       <x:c r="A160" s="14"/>
@@ -2279,6 +2440,7 @@
       <x:c r="H160" s="14"/>
       <x:c r="I160" s="14"/>
       <x:c r="J160" s="14"/>
+      <x:c r="K160" s="14"/>
     </x:row>
     <x:row r="161" ht="23" customHeight="1">
       <x:c r="A161" s="14"/>
@@ -2291,6 +2453,7 @@
       <x:c r="H161" s="14"/>
       <x:c r="I161" s="14"/>
       <x:c r="J161" s="14"/>
+      <x:c r="K161" s="14"/>
     </x:row>
     <x:row r="162" ht="23" customHeight="1">
       <x:c r="A162" s="14"/>
@@ -2303,6 +2466,7 @@
       <x:c r="H162" s="14"/>
       <x:c r="I162" s="14"/>
       <x:c r="J162" s="14"/>
+      <x:c r="K162" s="14"/>
     </x:row>
     <x:row r="163" ht="23" customHeight="1">
       <x:c r="A163" s="14"/>
@@ -2315,6 +2479,7 @@
       <x:c r="H163" s="14"/>
       <x:c r="I163" s="14"/>
       <x:c r="J163" s="14"/>
+      <x:c r="K163" s="14"/>
     </x:row>
     <x:row r="164" ht="23" customHeight="1">
       <x:c r="A164" s="14"/>
@@ -2327,6 +2492,7 @@
       <x:c r="H164" s="14"/>
       <x:c r="I164" s="14"/>
       <x:c r="J164" s="14"/>
+      <x:c r="K164" s="14"/>
     </x:row>
     <x:row r="165" ht="23" customHeight="1">
       <x:c r="A165" s="14"/>
@@ -2339,6 +2505,7 @@
       <x:c r="H165" s="14"/>
       <x:c r="I165" s="14"/>
       <x:c r="J165" s="14"/>
+      <x:c r="K165" s="14"/>
     </x:row>
     <x:row r="166" ht="23" customHeight="1">
       <x:c r="A166" s="14"/>
@@ -2351,6 +2518,7 @@
       <x:c r="H166" s="14"/>
       <x:c r="I166" s="14"/>
       <x:c r="J166" s="14"/>
+      <x:c r="K166" s="14"/>
     </x:row>
     <x:row r="167" ht="23" customHeight="1">
       <x:c r="A167" s="14"/>
@@ -2363,6 +2531,7 @@
       <x:c r="H167" s="14"/>
       <x:c r="I167" s="14"/>
       <x:c r="J167" s="14"/>
+      <x:c r="K167" s="14"/>
     </x:row>
     <x:row r="168" ht="23" customHeight="1">
       <x:c r="A168" s="14"/>
@@ -2375,6 +2544,7 @@
       <x:c r="H168" s="14"/>
       <x:c r="I168" s="14"/>
       <x:c r="J168" s="14"/>
+      <x:c r="K168" s="14"/>
     </x:row>
     <x:row r="169" ht="23" customHeight="1">
       <x:c r="A169" s="14"/>
@@ -2387,6 +2557,7 @@
       <x:c r="H169" s="14"/>
       <x:c r="I169" s="14"/>
       <x:c r="J169" s="14"/>
+      <x:c r="K169" s="14"/>
     </x:row>
     <x:row r="170" ht="23" customHeight="1">
       <x:c r="A170" s="14"/>
@@ -2399,6 +2570,7 @@
       <x:c r="H170" s="14"/>
       <x:c r="I170" s="14"/>
       <x:c r="J170" s="14"/>
+      <x:c r="K170" s="14"/>
     </x:row>
     <x:row r="171" ht="23" customHeight="1">
       <x:c r="A171" s="14"/>
@@ -2411,6 +2583,7 @@
       <x:c r="H171" s="14"/>
       <x:c r="I171" s="14"/>
       <x:c r="J171" s="14"/>
+      <x:c r="K171" s="14"/>
     </x:row>
     <x:row r="172" ht="23" customHeight="1">
       <x:c r="A172" s="14"/>
@@ -2423,6 +2596,7 @@
       <x:c r="H172" s="14"/>
       <x:c r="I172" s="14"/>
       <x:c r="J172" s="14"/>
+      <x:c r="K172" s="14"/>
     </x:row>
     <x:row r="173" ht="23" customHeight="1">
       <x:c r="A173" s="14"/>
@@ -2435,6 +2609,7 @@
       <x:c r="H173" s="14"/>
       <x:c r="I173" s="14"/>
       <x:c r="J173" s="14"/>
+      <x:c r="K173" s="14"/>
     </x:row>
     <x:row r="174" ht="23" customHeight="1">
       <x:c r="A174" s="14"/>
@@ -2447,6 +2622,7 @@
       <x:c r="H174" s="14"/>
       <x:c r="I174" s="14"/>
       <x:c r="J174" s="14"/>
+      <x:c r="K174" s="14"/>
     </x:row>
     <x:row r="175" ht="23" customHeight="1">
       <x:c r="A175" s="14"/>
@@ -2459,6 +2635,7 @@
       <x:c r="H175" s="14"/>
       <x:c r="I175" s="14"/>
       <x:c r="J175" s="14"/>
+      <x:c r="K175" s="14"/>
     </x:row>
     <x:row r="176" ht="23" customHeight="1">
       <x:c r="A176" s="14"/>
@@ -2471,6 +2648,7 @@
       <x:c r="H176" s="14"/>
       <x:c r="I176" s="14"/>
       <x:c r="J176" s="14"/>
+      <x:c r="K176" s="14"/>
     </x:row>
     <x:row r="177" ht="23" customHeight="1">
       <x:c r="A177" s="14"/>
@@ -2483,6 +2661,7 @@
       <x:c r="H177" s="14"/>
       <x:c r="I177" s="14"/>
       <x:c r="J177" s="14"/>
+      <x:c r="K177" s="14"/>
     </x:row>
     <x:row r="178" ht="23" customHeight="1">
       <x:c r="A178" s="14"/>
@@ -2495,6 +2674,7 @@
       <x:c r="H178" s="14"/>
       <x:c r="I178" s="14"/>
       <x:c r="J178" s="14"/>
+      <x:c r="K178" s="14"/>
     </x:row>
     <x:row r="179" ht="23" customHeight="1">
       <x:c r="A179" s="14"/>
@@ -2507,6 +2687,7 @@
       <x:c r="H179" s="14"/>
       <x:c r="I179" s="14"/>
       <x:c r="J179" s="14"/>
+      <x:c r="K179" s="14"/>
     </x:row>
     <x:row r="180" ht="23" customHeight="1">
       <x:c r="A180" s="14"/>
@@ -2519,6 +2700,7 @@
       <x:c r="H180" s="14"/>
       <x:c r="I180" s="14"/>
       <x:c r="J180" s="14"/>
+      <x:c r="K180" s="14"/>
     </x:row>
     <x:row r="181" ht="23" customHeight="1">
       <x:c r="A181" s="14"/>
@@ -2531,6 +2713,7 @@
       <x:c r="H181" s="14"/>
       <x:c r="I181" s="14"/>
       <x:c r="J181" s="14"/>
+      <x:c r="K181" s="14"/>
     </x:row>
     <x:row r="182" ht="23" customHeight="1">
       <x:c r="A182" s="14"/>
@@ -2543,6 +2726,7 @@
       <x:c r="H182" s="14"/>
       <x:c r="I182" s="14"/>
       <x:c r="J182" s="14"/>
+      <x:c r="K182" s="14"/>
     </x:row>
     <x:row r="183" ht="23" customHeight="1">
       <x:c r="A183" s="14"/>
@@ -2555,6 +2739,7 @@
       <x:c r="H183" s="14"/>
       <x:c r="I183" s="14"/>
       <x:c r="J183" s="14"/>
+      <x:c r="K183" s="14"/>
     </x:row>
     <x:row r="184" ht="23" customHeight="1">
       <x:c r="A184" s="14"/>
@@ -2567,6 +2752,7 @@
       <x:c r="H184" s="14"/>
       <x:c r="I184" s="14"/>
       <x:c r="J184" s="14"/>
+      <x:c r="K184" s="14"/>
     </x:row>
     <x:row r="185" ht="23" customHeight="1">
       <x:c r="A185" s="14"/>
@@ -2579,6 +2765,7 @@
       <x:c r="H185" s="14"/>
       <x:c r="I185" s="14"/>
       <x:c r="J185" s="14"/>
+      <x:c r="K185" s="14"/>
     </x:row>
     <x:row r="186" ht="23" customHeight="1">
       <x:c r="A186" s="14"/>
@@ -2591,6 +2778,7 @@
       <x:c r="H186" s="14"/>
       <x:c r="I186" s="14"/>
       <x:c r="J186" s="14"/>
+      <x:c r="K186" s="14"/>
     </x:row>
     <x:row r="187" ht="23" customHeight="1">
       <x:c r="A187" s="14"/>
@@ -2603,6 +2791,7 @@
       <x:c r="H187" s="14"/>
       <x:c r="I187" s="14"/>
       <x:c r="J187" s="14"/>
+      <x:c r="K187" s="14"/>
     </x:row>
     <x:row r="188" ht="23" customHeight="1">
       <x:c r="A188" s="14"/>
@@ -2615,6 +2804,7 @@
       <x:c r="H188" s="14"/>
       <x:c r="I188" s="14"/>
       <x:c r="J188" s="14"/>
+      <x:c r="K188" s="14"/>
     </x:row>
     <x:row r="189" ht="23" customHeight="1">
       <x:c r="A189" s="14"/>
@@ -2627,6 +2817,7 @@
       <x:c r="H189" s="14"/>
       <x:c r="I189" s="14"/>
       <x:c r="J189" s="14"/>
+      <x:c r="K189" s="14"/>
     </x:row>
     <x:row r="190" ht="23" customHeight="1">
       <x:c r="A190" s="14"/>
@@ -2639,6 +2830,7 @@
       <x:c r="H190" s="14"/>
       <x:c r="I190" s="14"/>
       <x:c r="J190" s="14"/>
+      <x:c r="K190" s="14"/>
     </x:row>
     <x:row r="191" ht="23" customHeight="1">
       <x:c r="A191" s="14"/>
@@ -2651,6 +2843,7 @@
       <x:c r="H191" s="14"/>
       <x:c r="I191" s="14"/>
       <x:c r="J191" s="14"/>
+      <x:c r="K191" s="14"/>
     </x:row>
     <x:row r="192" ht="23" customHeight="1">
       <x:c r="A192" s="14"/>
@@ -2663,6 +2856,7 @@
       <x:c r="H192" s="14"/>
       <x:c r="I192" s="14"/>
       <x:c r="J192" s="14"/>
+      <x:c r="K192" s="14"/>
     </x:row>
     <x:row r="193" ht="23" customHeight="1">
       <x:c r="A193" s="14"/>
@@ -2675,6 +2869,7 @@
       <x:c r="H193" s="14"/>
       <x:c r="I193" s="14"/>
       <x:c r="J193" s="14"/>
+      <x:c r="K193" s="14"/>
     </x:row>
     <x:row r="194" ht="23" customHeight="1">
       <x:c r="A194" s="14"/>
@@ -2687,6 +2882,7 @@
       <x:c r="H194" s="14"/>
       <x:c r="I194" s="14"/>
       <x:c r="J194" s="14"/>
+      <x:c r="K194" s="14"/>
     </x:row>
     <x:row r="195" ht="23" customHeight="1">
       <x:c r="A195" s="14"/>
@@ -2699,6 +2895,7 @@
       <x:c r="H195" s="14"/>
       <x:c r="I195" s="14"/>
       <x:c r="J195" s="14"/>
+      <x:c r="K195" s="14"/>
     </x:row>
     <x:row r="196" ht="23" customHeight="1">
       <x:c r="A196" s="14"/>
@@ -2711,6 +2908,7 @@
       <x:c r="H196" s="14"/>
       <x:c r="I196" s="14"/>
       <x:c r="J196" s="14"/>
+      <x:c r="K196" s="14"/>
     </x:row>
     <x:row r="197" ht="23" customHeight="1">
       <x:c r="A197" s="14"/>
@@ -2723,6 +2921,7 @@
       <x:c r="H197" s="14"/>
       <x:c r="I197" s="14"/>
       <x:c r="J197" s="14"/>
+      <x:c r="K197" s="14"/>
     </x:row>
     <x:row r="198" ht="23" customHeight="1">
       <x:c r="A198" s="14"/>
@@ -2735,6 +2934,7 @@
       <x:c r="H198" s="14"/>
       <x:c r="I198" s="14"/>
       <x:c r="J198" s="14"/>
+      <x:c r="K198" s="14"/>
     </x:row>
     <x:row r="199" ht="23" customHeight="1">
       <x:c r="A199" s="14"/>
@@ -2747,6 +2947,7 @@
       <x:c r="H199" s="14"/>
       <x:c r="I199" s="14"/>
       <x:c r="J199" s="14"/>
+      <x:c r="K199" s="14"/>
     </x:row>
     <x:row r="200" ht="23" customHeight="1">
       <x:c r="A200" s="14"/>
@@ -2759,6 +2960,7 @@
       <x:c r="H200" s="14"/>
       <x:c r="I200" s="14"/>
       <x:c r="J200" s="14"/>
+      <x:c r="K200" s="14"/>
     </x:row>
     <x:row r="201" ht="23" customHeight="1">
       <x:c r="A201" s="14"/>
@@ -2771,6 +2973,7 @@
       <x:c r="H201" s="14"/>
       <x:c r="I201" s="14"/>
       <x:c r="J201" s="14"/>
+      <x:c r="K201" s="14"/>
     </x:row>
     <x:row r="202" ht="23" customHeight="1">
       <x:c r="A202" s="14"/>
@@ -2783,6 +2986,7 @@
       <x:c r="H202" s="14"/>
       <x:c r="I202" s="14"/>
       <x:c r="J202" s="14"/>
+      <x:c r="K202" s="14"/>
     </x:row>
     <x:row r="203" ht="23" customHeight="1">
       <x:c r="A203" s="14"/>
@@ -2795,6 +2999,7 @@
       <x:c r="H203" s="14"/>
       <x:c r="I203" s="14"/>
       <x:c r="J203" s="14"/>
+      <x:c r="K203" s="14"/>
     </x:row>
     <x:row r="204" ht="23" customHeight="1">
       <x:c r="A204" s="14"/>
@@ -2807,6 +3012,7 @@
       <x:c r="H204" s="14"/>
       <x:c r="I204" s="14"/>
       <x:c r="J204" s="14"/>
+      <x:c r="K204" s="14"/>
     </x:row>
     <x:row r="205" ht="23" customHeight="1">
       <x:c r="A205" s="14"/>
@@ -2819,6 +3025,7 @@
       <x:c r="H205" s="14"/>
       <x:c r="I205" s="14"/>
       <x:c r="J205" s="14"/>
+      <x:c r="K205" s="14"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">

</xml_diff>

<commit_message>
fix: address round-2 review (exclude demo copy from venue backfill, drop description columns from import template, admin email fixes)
</commit_message>
<xml_diff>
--- a/public/session-import-template.xlsx
+++ b/public/session-import-template.xlsx
@@ -341,10 +341,8 @@
     <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="30" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="38" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="38" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="23" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="24" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="23" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -358,9 +356,7 @@
       <x:c r="F1" s="1"/>
       <x:c r="G1" s="1"/>
       <x:c r="H1" s="1"/>
-      <x:c r="I1" s="1"/>
-      <x:c r="J1" s="1"/>
-      <x:c r="K1" s="14"/>
+      <x:c r="I1" s="14"/>
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
       <x:c r="A2" s="2" t="str">
@@ -373,9 +369,7 @@
       <x:c r="F2" s="2"/>
       <x:c r="G2" s="2"/>
       <x:c r="H2" s="2"/>
-      <x:c r="I2" s="2"/>
-      <x:c r="J2" s="2"/>
-      <x:c r="K2" s="14"/>
+      <x:c r="I2" s="14"/>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
       <x:c r="A3" s="2" t="str">
@@ -388,9 +382,7 @@
       <x:c r="F3" s="2"/>
       <x:c r="G3" s="2"/>
       <x:c r="H3" s="2"/>
-      <x:c r="I3" s="2"/>
-      <x:c r="J3" s="2"/>
-      <x:c r="K3" s="14"/>
+      <x:c r="I3" s="14"/>
     </x:row>
     <x:row r="5" ht="42" customHeight="1">
       <x:c r="A5" s="13" t="str">
@@ -415,15 +407,9 @@
         <x:v>Formats (singles, doubles) / 形式</x:v>
       </x:c>
       <x:c r="H5" s="13" t="str">
-        <x:v>Description (English, optional) / 英文描述（可选）</x:v>
+        <x:v>Status (published, draft) / 状态</x:v>
       </x:c>
       <x:c r="I5" s="13" t="str">
-        <x:v>Description (Chinese, optional) / 中文描述（可选）</x:v>
-      </x:c>
-      <x:c r="J5" s="13" t="str">
-        <x:v>Status (published, draft) / 状态</x:v>
-      </x:c>
-      <x:c r="K5" s="13" t="str">
         <x:v>Seeking levels (1.0, 1.5) / 寻找水平</x:v>
       </x:c>
     </x:row>
@@ -437,8 +423,6 @@
       <x:c r="G6" s="14"/>
       <x:c r="H6" s="14"/>
       <x:c r="I6" s="14"/>
-      <x:c r="J6" s="14"/>
-      <x:c r="K6" s="14"/>
     </x:row>
     <x:row r="7" ht="23" customHeight="1">
       <x:c r="A7" s="14"/>
@@ -450,8 +434,6 @@
       <x:c r="G7" s="14"/>
       <x:c r="H7" s="14"/>
       <x:c r="I7" s="14"/>
-      <x:c r="J7" s="14"/>
-      <x:c r="K7" s="14"/>
     </x:row>
     <x:row r="8" ht="23" customHeight="1">
       <x:c r="A8" s="14"/>
@@ -463,8 +445,6 @@
       <x:c r="G8" s="14"/>
       <x:c r="H8" s="14"/>
       <x:c r="I8" s="14"/>
-      <x:c r="J8" s="14"/>
-      <x:c r="K8" s="14"/>
     </x:row>
     <x:row r="9" ht="23" customHeight="1">
       <x:c r="A9" s="14"/>
@@ -476,8 +456,6 @@
       <x:c r="G9" s="14"/>
       <x:c r="H9" s="14"/>
       <x:c r="I9" s="14"/>
-      <x:c r="J9" s="14"/>
-      <x:c r="K9" s="14"/>
     </x:row>
     <x:row r="10" ht="23" customHeight="1">
       <x:c r="A10" s="14"/>
@@ -489,8 +467,6 @@
       <x:c r="G10" s="14"/>
       <x:c r="H10" s="14"/>
       <x:c r="I10" s="14"/>
-      <x:c r="J10" s="14"/>
-      <x:c r="K10" s="14"/>
     </x:row>
     <x:row r="11" ht="23" customHeight="1">
       <x:c r="A11" s="14"/>
@@ -502,8 +478,6 @@
       <x:c r="G11" s="14"/>
       <x:c r="H11" s="14"/>
       <x:c r="I11" s="14"/>
-      <x:c r="J11" s="14"/>
-      <x:c r="K11" s="14"/>
     </x:row>
     <x:row r="12" ht="23" customHeight="1">
       <x:c r="A12" s="14"/>
@@ -515,8 +489,6 @@
       <x:c r="G12" s="14"/>
       <x:c r="H12" s="14"/>
       <x:c r="I12" s="14"/>
-      <x:c r="J12" s="14"/>
-      <x:c r="K12" s="14"/>
     </x:row>
     <x:row r="13" ht="23" customHeight="1">
       <x:c r="A13" s="14"/>
@@ -528,8 +500,6 @@
       <x:c r="G13" s="14"/>
       <x:c r="H13" s="14"/>
       <x:c r="I13" s="14"/>
-      <x:c r="J13" s="14"/>
-      <x:c r="K13" s="14"/>
     </x:row>
     <x:row r="14" ht="23" customHeight="1">
       <x:c r="A14" s="14"/>
@@ -541,8 +511,6 @@
       <x:c r="G14" s="14"/>
       <x:c r="H14" s="14"/>
       <x:c r="I14" s="14"/>
-      <x:c r="J14" s="14"/>
-      <x:c r="K14" s="14"/>
     </x:row>
     <x:row r="15" ht="23" customHeight="1">
       <x:c r="A15" s="14"/>
@@ -554,8 +522,6 @@
       <x:c r="G15" s="14"/>
       <x:c r="H15" s="14"/>
       <x:c r="I15" s="14"/>
-      <x:c r="J15" s="14"/>
-      <x:c r="K15" s="14"/>
     </x:row>
     <x:row r="16" ht="23" customHeight="1">
       <x:c r="A16" s="14"/>
@@ -567,8 +533,6 @@
       <x:c r="G16" s="14"/>
       <x:c r="H16" s="14"/>
       <x:c r="I16" s="14"/>
-      <x:c r="J16" s="14"/>
-      <x:c r="K16" s="14"/>
     </x:row>
     <x:row r="17" ht="23" customHeight="1">
       <x:c r="A17" s="14"/>
@@ -580,8 +544,6 @@
       <x:c r="G17" s="14"/>
       <x:c r="H17" s="14"/>
       <x:c r="I17" s="14"/>
-      <x:c r="J17" s="14"/>
-      <x:c r="K17" s="14"/>
     </x:row>
     <x:row r="18" ht="23" customHeight="1">
       <x:c r="A18" s="14"/>
@@ -593,8 +555,6 @@
       <x:c r="G18" s="14"/>
       <x:c r="H18" s="14"/>
       <x:c r="I18" s="14"/>
-      <x:c r="J18" s="14"/>
-      <x:c r="K18" s="14"/>
     </x:row>
     <x:row r="19" ht="23" customHeight="1">
       <x:c r="A19" s="14"/>
@@ -606,8 +566,6 @@
       <x:c r="G19" s="14"/>
       <x:c r="H19" s="14"/>
       <x:c r="I19" s="14"/>
-      <x:c r="J19" s="14"/>
-      <x:c r="K19" s="14"/>
     </x:row>
     <x:row r="20" ht="23" customHeight="1">
       <x:c r="A20" s="14"/>
@@ -619,8 +577,6 @@
       <x:c r="G20" s="14"/>
       <x:c r="H20" s="14"/>
       <x:c r="I20" s="14"/>
-      <x:c r="J20" s="14"/>
-      <x:c r="K20" s="14"/>
     </x:row>
     <x:row r="21" ht="23" customHeight="1">
       <x:c r="A21" s="14"/>
@@ -632,8 +588,6 @@
       <x:c r="G21" s="14"/>
       <x:c r="H21" s="14"/>
       <x:c r="I21" s="14"/>
-      <x:c r="J21" s="14"/>
-      <x:c r="K21" s="14"/>
     </x:row>
     <x:row r="22" ht="23" customHeight="1">
       <x:c r="A22" s="14"/>
@@ -645,8 +599,6 @@
       <x:c r="G22" s="14"/>
       <x:c r="H22" s="14"/>
       <x:c r="I22" s="14"/>
-      <x:c r="J22" s="14"/>
-      <x:c r="K22" s="14"/>
     </x:row>
     <x:row r="23" ht="23" customHeight="1">
       <x:c r="A23" s="14"/>
@@ -658,8 +610,6 @@
       <x:c r="G23" s="14"/>
       <x:c r="H23" s="14"/>
       <x:c r="I23" s="14"/>
-      <x:c r="J23" s="14"/>
-      <x:c r="K23" s="14"/>
     </x:row>
     <x:row r="24" ht="23" customHeight="1">
       <x:c r="A24" s="14"/>
@@ -671,8 +621,6 @@
       <x:c r="G24" s="14"/>
       <x:c r="H24" s="14"/>
       <x:c r="I24" s="14"/>
-      <x:c r="J24" s="14"/>
-      <x:c r="K24" s="14"/>
     </x:row>
     <x:row r="25" ht="23" customHeight="1">
       <x:c r="A25" s="14"/>
@@ -684,8 +632,6 @@
       <x:c r="G25" s="14"/>
       <x:c r="H25" s="14"/>
       <x:c r="I25" s="14"/>
-      <x:c r="J25" s="14"/>
-      <x:c r="K25" s="14"/>
     </x:row>
     <x:row r="26" ht="23" customHeight="1">
       <x:c r="A26" s="14"/>
@@ -697,8 +643,6 @@
       <x:c r="G26" s="14"/>
       <x:c r="H26" s="14"/>
       <x:c r="I26" s="14"/>
-      <x:c r="J26" s="14"/>
-      <x:c r="K26" s="14"/>
     </x:row>
     <x:row r="27" ht="23" customHeight="1">
       <x:c r="A27" s="14"/>
@@ -710,8 +654,6 @@
       <x:c r="G27" s="14"/>
       <x:c r="H27" s="14"/>
       <x:c r="I27" s="14"/>
-      <x:c r="J27" s="14"/>
-      <x:c r="K27" s="14"/>
     </x:row>
     <x:row r="28" ht="23" customHeight="1">
       <x:c r="A28" s="14"/>
@@ -723,8 +665,6 @@
       <x:c r="G28" s="14"/>
       <x:c r="H28" s="14"/>
       <x:c r="I28" s="14"/>
-      <x:c r="J28" s="14"/>
-      <x:c r="K28" s="14"/>
     </x:row>
     <x:row r="29" ht="23" customHeight="1">
       <x:c r="A29" s="14"/>
@@ -736,8 +676,6 @@
       <x:c r="G29" s="14"/>
       <x:c r="H29" s="14"/>
       <x:c r="I29" s="14"/>
-      <x:c r="J29" s="14"/>
-      <x:c r="K29" s="14"/>
     </x:row>
     <x:row r="30" ht="23" customHeight="1">
       <x:c r="A30" s="14"/>
@@ -749,8 +687,6 @@
       <x:c r="G30" s="14"/>
       <x:c r="H30" s="14"/>
       <x:c r="I30" s="14"/>
-      <x:c r="J30" s="14"/>
-      <x:c r="K30" s="14"/>
     </x:row>
     <x:row r="31" ht="23" customHeight="1">
       <x:c r="A31" s="14"/>
@@ -762,8 +698,6 @@
       <x:c r="G31" s="14"/>
       <x:c r="H31" s="14"/>
       <x:c r="I31" s="14"/>
-      <x:c r="J31" s="14"/>
-      <x:c r="K31" s="14"/>
     </x:row>
     <x:row r="32" ht="23" customHeight="1">
       <x:c r="A32" s="14"/>
@@ -775,8 +709,6 @@
       <x:c r="G32" s="14"/>
       <x:c r="H32" s="14"/>
       <x:c r="I32" s="14"/>
-      <x:c r="J32" s="14"/>
-      <x:c r="K32" s="14"/>
     </x:row>
     <x:row r="33" ht="23" customHeight="1">
       <x:c r="A33" s="14"/>
@@ -788,8 +720,6 @@
       <x:c r="G33" s="14"/>
       <x:c r="H33" s="14"/>
       <x:c r="I33" s="14"/>
-      <x:c r="J33" s="14"/>
-      <x:c r="K33" s="14"/>
     </x:row>
     <x:row r="34" ht="23" customHeight="1">
       <x:c r="A34" s="14"/>
@@ -801,8 +731,6 @@
       <x:c r="G34" s="14"/>
       <x:c r="H34" s="14"/>
       <x:c r="I34" s="14"/>
-      <x:c r="J34" s="14"/>
-      <x:c r="K34" s="14"/>
     </x:row>
     <x:row r="35" ht="23" customHeight="1">
       <x:c r="A35" s="14"/>
@@ -814,8 +742,6 @@
       <x:c r="G35" s="14"/>
       <x:c r="H35" s="14"/>
       <x:c r="I35" s="14"/>
-      <x:c r="J35" s="14"/>
-      <x:c r="K35" s="14"/>
     </x:row>
     <x:row r="36" ht="23" customHeight="1">
       <x:c r="A36" s="14"/>
@@ -827,8 +753,6 @@
       <x:c r="G36" s="14"/>
       <x:c r="H36" s="14"/>
       <x:c r="I36" s="14"/>
-      <x:c r="J36" s="14"/>
-      <x:c r="K36" s="14"/>
     </x:row>
     <x:row r="37" ht="23" customHeight="1">
       <x:c r="A37" s="14"/>
@@ -840,8 +764,6 @@
       <x:c r="G37" s="14"/>
       <x:c r="H37" s="14"/>
       <x:c r="I37" s="14"/>
-      <x:c r="J37" s="14"/>
-      <x:c r="K37" s="14"/>
     </x:row>
     <x:row r="38" ht="23" customHeight="1">
       <x:c r="A38" s="14"/>
@@ -853,8 +775,6 @@
       <x:c r="G38" s="14"/>
       <x:c r="H38" s="14"/>
       <x:c r="I38" s="14"/>
-      <x:c r="J38" s="14"/>
-      <x:c r="K38" s="14"/>
     </x:row>
     <x:row r="39" ht="23" customHeight="1">
       <x:c r="A39" s="14"/>
@@ -866,8 +786,6 @@
       <x:c r="G39" s="14"/>
       <x:c r="H39" s="14"/>
       <x:c r="I39" s="14"/>
-      <x:c r="J39" s="14"/>
-      <x:c r="K39" s="14"/>
     </x:row>
     <x:row r="40" ht="23" customHeight="1">
       <x:c r="A40" s="14"/>
@@ -879,8 +797,6 @@
       <x:c r="G40" s="14"/>
       <x:c r="H40" s="14"/>
       <x:c r="I40" s="14"/>
-      <x:c r="J40" s="14"/>
-      <x:c r="K40" s="14"/>
     </x:row>
     <x:row r="41" ht="23" customHeight="1">
       <x:c r="A41" s="14"/>
@@ -892,8 +808,6 @@
       <x:c r="G41" s="14"/>
       <x:c r="H41" s="14"/>
       <x:c r="I41" s="14"/>
-      <x:c r="J41" s="14"/>
-      <x:c r="K41" s="14"/>
     </x:row>
     <x:row r="42" ht="23" customHeight="1">
       <x:c r="A42" s="14"/>
@@ -905,8 +819,6 @@
       <x:c r="G42" s="14"/>
       <x:c r="H42" s="14"/>
       <x:c r="I42" s="14"/>
-      <x:c r="J42" s="14"/>
-      <x:c r="K42" s="14"/>
     </x:row>
     <x:row r="43" ht="23" customHeight="1">
       <x:c r="A43" s="14"/>
@@ -918,8 +830,6 @@
       <x:c r="G43" s="14"/>
       <x:c r="H43" s="14"/>
       <x:c r="I43" s="14"/>
-      <x:c r="J43" s="14"/>
-      <x:c r="K43" s="14"/>
     </x:row>
     <x:row r="44" ht="23" customHeight="1">
       <x:c r="A44" s="14"/>
@@ -931,8 +841,6 @@
       <x:c r="G44" s="14"/>
       <x:c r="H44" s="14"/>
       <x:c r="I44" s="14"/>
-      <x:c r="J44" s="14"/>
-      <x:c r="K44" s="14"/>
     </x:row>
     <x:row r="45" ht="23" customHeight="1">
       <x:c r="A45" s="14"/>
@@ -944,8 +852,6 @@
       <x:c r="G45" s="14"/>
       <x:c r="H45" s="14"/>
       <x:c r="I45" s="14"/>
-      <x:c r="J45" s="14"/>
-      <x:c r="K45" s="14"/>
     </x:row>
     <x:row r="46" ht="23" customHeight="1">
       <x:c r="A46" s="14"/>
@@ -957,8 +863,6 @@
       <x:c r="G46" s="14"/>
       <x:c r="H46" s="14"/>
       <x:c r="I46" s="14"/>
-      <x:c r="J46" s="14"/>
-      <x:c r="K46" s="14"/>
     </x:row>
     <x:row r="47" ht="23" customHeight="1">
       <x:c r="A47" s="14"/>
@@ -970,8 +874,6 @@
       <x:c r="G47" s="14"/>
       <x:c r="H47" s="14"/>
       <x:c r="I47" s="14"/>
-      <x:c r="J47" s="14"/>
-      <x:c r="K47" s="14"/>
     </x:row>
     <x:row r="48" ht="23" customHeight="1">
       <x:c r="A48" s="14"/>
@@ -983,8 +885,6 @@
       <x:c r="G48" s="14"/>
       <x:c r="H48" s="14"/>
       <x:c r="I48" s="14"/>
-      <x:c r="J48" s="14"/>
-      <x:c r="K48" s="14"/>
     </x:row>
     <x:row r="49" ht="23" customHeight="1">
       <x:c r="A49" s="14"/>
@@ -996,8 +896,6 @@
       <x:c r="G49" s="14"/>
       <x:c r="H49" s="14"/>
       <x:c r="I49" s="14"/>
-      <x:c r="J49" s="14"/>
-      <x:c r="K49" s="14"/>
     </x:row>
     <x:row r="50" ht="23" customHeight="1">
       <x:c r="A50" s="14"/>
@@ -1009,8 +907,6 @@
       <x:c r="G50" s="14"/>
       <x:c r="H50" s="14"/>
       <x:c r="I50" s="14"/>
-      <x:c r="J50" s="14"/>
-      <x:c r="K50" s="14"/>
     </x:row>
     <x:row r="51" ht="23" customHeight="1">
       <x:c r="A51" s="14"/>
@@ -1022,8 +918,6 @@
       <x:c r="G51" s="14"/>
       <x:c r="H51" s="14"/>
       <x:c r="I51" s="14"/>
-      <x:c r="J51" s="14"/>
-      <x:c r="K51" s="14"/>
     </x:row>
     <x:row r="52" ht="23" customHeight="1">
       <x:c r="A52" s="14"/>
@@ -1035,8 +929,6 @@
       <x:c r="G52" s="14"/>
       <x:c r="H52" s="14"/>
       <x:c r="I52" s="14"/>
-      <x:c r="J52" s="14"/>
-      <x:c r="K52" s="14"/>
     </x:row>
     <x:row r="53" ht="23" customHeight="1">
       <x:c r="A53" s="14"/>
@@ -1048,8 +940,6 @@
       <x:c r="G53" s="14"/>
       <x:c r="H53" s="14"/>
       <x:c r="I53" s="14"/>
-      <x:c r="J53" s="14"/>
-      <x:c r="K53" s="14"/>
     </x:row>
     <x:row r="54" ht="23" customHeight="1">
       <x:c r="A54" s="14"/>
@@ -1061,8 +951,6 @@
       <x:c r="G54" s="14"/>
       <x:c r="H54" s="14"/>
       <x:c r="I54" s="14"/>
-      <x:c r="J54" s="14"/>
-      <x:c r="K54" s="14"/>
     </x:row>
     <x:row r="55" ht="23" customHeight="1">
       <x:c r="A55" s="14"/>
@@ -1074,8 +962,6 @@
       <x:c r="G55" s="14"/>
       <x:c r="H55" s="14"/>
       <x:c r="I55" s="14"/>
-      <x:c r="J55" s="14"/>
-      <x:c r="K55" s="14"/>
     </x:row>
     <x:row r="56" ht="23" customHeight="1">
       <x:c r="A56" s="14"/>
@@ -1087,8 +973,6 @@
       <x:c r="G56" s="14"/>
       <x:c r="H56" s="14"/>
       <x:c r="I56" s="14"/>
-      <x:c r="J56" s="14"/>
-      <x:c r="K56" s="14"/>
     </x:row>
     <x:row r="57" ht="23" customHeight="1">
       <x:c r="A57" s="14"/>
@@ -1100,8 +984,6 @@
       <x:c r="G57" s="14"/>
       <x:c r="H57" s="14"/>
       <x:c r="I57" s="14"/>
-      <x:c r="J57" s="14"/>
-      <x:c r="K57" s="14"/>
     </x:row>
     <x:row r="58" ht="23" customHeight="1">
       <x:c r="A58" s="14"/>
@@ -1113,8 +995,6 @@
       <x:c r="G58" s="14"/>
       <x:c r="H58" s="14"/>
       <x:c r="I58" s="14"/>
-      <x:c r="J58" s="14"/>
-      <x:c r="K58" s="14"/>
     </x:row>
     <x:row r="59" ht="23" customHeight="1">
       <x:c r="A59" s="14"/>
@@ -1126,8 +1006,6 @@
       <x:c r="G59" s="14"/>
       <x:c r="H59" s="14"/>
       <x:c r="I59" s="14"/>
-      <x:c r="J59" s="14"/>
-      <x:c r="K59" s="14"/>
     </x:row>
     <x:row r="60" ht="23" customHeight="1">
       <x:c r="A60" s="14"/>
@@ -1139,8 +1017,6 @@
       <x:c r="G60" s="14"/>
       <x:c r="H60" s="14"/>
       <x:c r="I60" s="14"/>
-      <x:c r="J60" s="14"/>
-      <x:c r="K60" s="14"/>
     </x:row>
     <x:row r="61" ht="23" customHeight="1">
       <x:c r="A61" s="14"/>
@@ -1152,8 +1028,6 @@
       <x:c r="G61" s="14"/>
       <x:c r="H61" s="14"/>
       <x:c r="I61" s="14"/>
-      <x:c r="J61" s="14"/>
-      <x:c r="K61" s="14"/>
     </x:row>
     <x:row r="62" ht="23" customHeight="1">
       <x:c r="A62" s="14"/>
@@ -1165,8 +1039,6 @@
       <x:c r="G62" s="14"/>
       <x:c r="H62" s="14"/>
       <x:c r="I62" s="14"/>
-      <x:c r="J62" s="14"/>
-      <x:c r="K62" s="14"/>
     </x:row>
     <x:row r="63" ht="23" customHeight="1">
       <x:c r="A63" s="14"/>
@@ -1178,8 +1050,6 @@
       <x:c r="G63" s="14"/>
       <x:c r="H63" s="14"/>
       <x:c r="I63" s="14"/>
-      <x:c r="J63" s="14"/>
-      <x:c r="K63" s="14"/>
     </x:row>
     <x:row r="64" ht="23" customHeight="1">
       <x:c r="A64" s="14"/>
@@ -1191,8 +1061,6 @@
       <x:c r="G64" s="14"/>
       <x:c r="H64" s="14"/>
       <x:c r="I64" s="14"/>
-      <x:c r="J64" s="14"/>
-      <x:c r="K64" s="14"/>
     </x:row>
     <x:row r="65" ht="23" customHeight="1">
       <x:c r="A65" s="14"/>
@@ -1204,8 +1072,6 @@
       <x:c r="G65" s="14"/>
       <x:c r="H65" s="14"/>
       <x:c r="I65" s="14"/>
-      <x:c r="J65" s="14"/>
-      <x:c r="K65" s="14"/>
     </x:row>
     <x:row r="66" ht="23" customHeight="1">
       <x:c r="A66" s="14"/>
@@ -1217,8 +1083,6 @@
       <x:c r="G66" s="14"/>
       <x:c r="H66" s="14"/>
       <x:c r="I66" s="14"/>
-      <x:c r="J66" s="14"/>
-      <x:c r="K66" s="14"/>
     </x:row>
     <x:row r="67" ht="23" customHeight="1">
       <x:c r="A67" s="14"/>
@@ -1230,8 +1094,6 @@
       <x:c r="G67" s="14"/>
       <x:c r="H67" s="14"/>
       <x:c r="I67" s="14"/>
-      <x:c r="J67" s="14"/>
-      <x:c r="K67" s="14"/>
     </x:row>
     <x:row r="68" ht="23" customHeight="1">
       <x:c r="A68" s="14"/>
@@ -1243,8 +1105,6 @@
       <x:c r="G68" s="14"/>
       <x:c r="H68" s="14"/>
       <x:c r="I68" s="14"/>
-      <x:c r="J68" s="14"/>
-      <x:c r="K68" s="14"/>
     </x:row>
     <x:row r="69" ht="23" customHeight="1">
       <x:c r="A69" s="14"/>
@@ -1256,8 +1116,6 @@
       <x:c r="G69" s="14"/>
       <x:c r="H69" s="14"/>
       <x:c r="I69" s="14"/>
-      <x:c r="J69" s="14"/>
-      <x:c r="K69" s="14"/>
     </x:row>
     <x:row r="70" ht="23" customHeight="1">
       <x:c r="A70" s="14"/>
@@ -1269,8 +1127,6 @@
       <x:c r="G70" s="14"/>
       <x:c r="H70" s="14"/>
       <x:c r="I70" s="14"/>
-      <x:c r="J70" s="14"/>
-      <x:c r="K70" s="14"/>
     </x:row>
     <x:row r="71" ht="23" customHeight="1">
       <x:c r="A71" s="14"/>
@@ -1282,8 +1138,6 @@
       <x:c r="G71" s="14"/>
       <x:c r="H71" s="14"/>
       <x:c r="I71" s="14"/>
-      <x:c r="J71" s="14"/>
-      <x:c r="K71" s="14"/>
     </x:row>
     <x:row r="72" ht="23" customHeight="1">
       <x:c r="A72" s="14"/>
@@ -1295,8 +1149,6 @@
       <x:c r="G72" s="14"/>
       <x:c r="H72" s="14"/>
       <x:c r="I72" s="14"/>
-      <x:c r="J72" s="14"/>
-      <x:c r="K72" s="14"/>
     </x:row>
     <x:row r="73" ht="23" customHeight="1">
       <x:c r="A73" s="14"/>
@@ -1308,8 +1160,6 @@
       <x:c r="G73" s="14"/>
       <x:c r="H73" s="14"/>
       <x:c r="I73" s="14"/>
-      <x:c r="J73" s="14"/>
-      <x:c r="K73" s="14"/>
     </x:row>
     <x:row r="74" ht="23" customHeight="1">
       <x:c r="A74" s="14"/>
@@ -1321,8 +1171,6 @@
       <x:c r="G74" s="14"/>
       <x:c r="H74" s="14"/>
       <x:c r="I74" s="14"/>
-      <x:c r="J74" s="14"/>
-      <x:c r="K74" s="14"/>
     </x:row>
     <x:row r="75" ht="23" customHeight="1">
       <x:c r="A75" s="14"/>
@@ -1334,8 +1182,6 @@
       <x:c r="G75" s="14"/>
       <x:c r="H75" s="14"/>
       <x:c r="I75" s="14"/>
-      <x:c r="J75" s="14"/>
-      <x:c r="K75" s="14"/>
     </x:row>
     <x:row r="76" ht="23" customHeight="1">
       <x:c r="A76" s="14"/>
@@ -1347,8 +1193,6 @@
       <x:c r="G76" s="14"/>
       <x:c r="H76" s="14"/>
       <x:c r="I76" s="14"/>
-      <x:c r="J76" s="14"/>
-      <x:c r="K76" s="14"/>
     </x:row>
     <x:row r="77" ht="23" customHeight="1">
       <x:c r="A77" s="14"/>
@@ -1360,8 +1204,6 @@
       <x:c r="G77" s="14"/>
       <x:c r="H77" s="14"/>
       <x:c r="I77" s="14"/>
-      <x:c r="J77" s="14"/>
-      <x:c r="K77" s="14"/>
     </x:row>
     <x:row r="78" ht="23" customHeight="1">
       <x:c r="A78" s="14"/>
@@ -1373,8 +1215,6 @@
       <x:c r="G78" s="14"/>
       <x:c r="H78" s="14"/>
       <x:c r="I78" s="14"/>
-      <x:c r="J78" s="14"/>
-      <x:c r="K78" s="14"/>
     </x:row>
     <x:row r="79" ht="23" customHeight="1">
       <x:c r="A79" s="14"/>
@@ -1386,8 +1226,6 @@
       <x:c r="G79" s="14"/>
       <x:c r="H79" s="14"/>
       <x:c r="I79" s="14"/>
-      <x:c r="J79" s="14"/>
-      <x:c r="K79" s="14"/>
     </x:row>
     <x:row r="80" ht="23" customHeight="1">
       <x:c r="A80" s="14"/>
@@ -1399,8 +1237,6 @@
       <x:c r="G80" s="14"/>
       <x:c r="H80" s="14"/>
       <x:c r="I80" s="14"/>
-      <x:c r="J80" s="14"/>
-      <x:c r="K80" s="14"/>
     </x:row>
     <x:row r="81" ht="23" customHeight="1">
       <x:c r="A81" s="14"/>
@@ -1412,8 +1248,6 @@
       <x:c r="G81" s="14"/>
       <x:c r="H81" s="14"/>
       <x:c r="I81" s="14"/>
-      <x:c r="J81" s="14"/>
-      <x:c r="K81" s="14"/>
     </x:row>
     <x:row r="82" ht="23" customHeight="1">
       <x:c r="A82" s="14"/>
@@ -1425,8 +1259,6 @@
       <x:c r="G82" s="14"/>
       <x:c r="H82" s="14"/>
       <x:c r="I82" s="14"/>
-      <x:c r="J82" s="14"/>
-      <x:c r="K82" s="14"/>
     </x:row>
     <x:row r="83" ht="23" customHeight="1">
       <x:c r="A83" s="14"/>
@@ -1438,8 +1270,6 @@
       <x:c r="G83" s="14"/>
       <x:c r="H83" s="14"/>
       <x:c r="I83" s="14"/>
-      <x:c r="J83" s="14"/>
-      <x:c r="K83" s="14"/>
     </x:row>
     <x:row r="84" ht="23" customHeight="1">
       <x:c r="A84" s="14"/>
@@ -1451,8 +1281,6 @@
       <x:c r="G84" s="14"/>
       <x:c r="H84" s="14"/>
       <x:c r="I84" s="14"/>
-      <x:c r="J84" s="14"/>
-      <x:c r="K84" s="14"/>
     </x:row>
     <x:row r="85" ht="23" customHeight="1">
       <x:c r="A85" s="14"/>
@@ -1464,8 +1292,6 @@
       <x:c r="G85" s="14"/>
       <x:c r="H85" s="14"/>
       <x:c r="I85" s="14"/>
-      <x:c r="J85" s="14"/>
-      <x:c r="K85" s="14"/>
     </x:row>
     <x:row r="86" ht="23" customHeight="1">
       <x:c r="A86" s="14"/>
@@ -1477,8 +1303,6 @@
       <x:c r="G86" s="14"/>
       <x:c r="H86" s="14"/>
       <x:c r="I86" s="14"/>
-      <x:c r="J86" s="14"/>
-      <x:c r="K86" s="14"/>
     </x:row>
     <x:row r="87" ht="23" customHeight="1">
       <x:c r="A87" s="14"/>
@@ -1490,8 +1314,6 @@
       <x:c r="G87" s="14"/>
       <x:c r="H87" s="14"/>
       <x:c r="I87" s="14"/>
-      <x:c r="J87" s="14"/>
-      <x:c r="K87" s="14"/>
     </x:row>
     <x:row r="88" ht="23" customHeight="1">
       <x:c r="A88" s="14"/>
@@ -1503,8 +1325,6 @@
       <x:c r="G88" s="14"/>
       <x:c r="H88" s="14"/>
       <x:c r="I88" s="14"/>
-      <x:c r="J88" s="14"/>
-      <x:c r="K88" s="14"/>
     </x:row>
     <x:row r="89" ht="23" customHeight="1">
       <x:c r="A89" s="14"/>
@@ -1516,8 +1336,6 @@
       <x:c r="G89" s="14"/>
       <x:c r="H89" s="14"/>
       <x:c r="I89" s="14"/>
-      <x:c r="J89" s="14"/>
-      <x:c r="K89" s="14"/>
     </x:row>
     <x:row r="90" ht="23" customHeight="1">
       <x:c r="A90" s="14"/>
@@ -1529,8 +1347,6 @@
       <x:c r="G90" s="14"/>
       <x:c r="H90" s="14"/>
       <x:c r="I90" s="14"/>
-      <x:c r="J90" s="14"/>
-      <x:c r="K90" s="14"/>
     </x:row>
     <x:row r="91" ht="23" customHeight="1">
       <x:c r="A91" s="14"/>
@@ -1542,8 +1358,6 @@
       <x:c r="G91" s="14"/>
       <x:c r="H91" s="14"/>
       <x:c r="I91" s="14"/>
-      <x:c r="J91" s="14"/>
-      <x:c r="K91" s="14"/>
     </x:row>
     <x:row r="92" ht="23" customHeight="1">
       <x:c r="A92" s="14"/>
@@ -1555,8 +1369,6 @@
       <x:c r="G92" s="14"/>
       <x:c r="H92" s="14"/>
       <x:c r="I92" s="14"/>
-      <x:c r="J92" s="14"/>
-      <x:c r="K92" s="14"/>
     </x:row>
     <x:row r="93" ht="23" customHeight="1">
       <x:c r="A93" s="14"/>
@@ -1568,8 +1380,6 @@
       <x:c r="G93" s="14"/>
       <x:c r="H93" s="14"/>
       <x:c r="I93" s="14"/>
-      <x:c r="J93" s="14"/>
-      <x:c r="K93" s="14"/>
     </x:row>
     <x:row r="94" ht="23" customHeight="1">
       <x:c r="A94" s="14"/>
@@ -1581,8 +1391,6 @@
       <x:c r="G94" s="14"/>
       <x:c r="H94" s="14"/>
       <x:c r="I94" s="14"/>
-      <x:c r="J94" s="14"/>
-      <x:c r="K94" s="14"/>
     </x:row>
     <x:row r="95" ht="23" customHeight="1">
       <x:c r="A95" s="14"/>
@@ -1594,8 +1402,6 @@
       <x:c r="G95" s="14"/>
       <x:c r="H95" s="14"/>
       <x:c r="I95" s="14"/>
-      <x:c r="J95" s="14"/>
-      <x:c r="K95" s="14"/>
     </x:row>
     <x:row r="96" ht="23" customHeight="1">
       <x:c r="A96" s="14"/>
@@ -1607,8 +1413,6 @@
       <x:c r="G96" s="14"/>
       <x:c r="H96" s="14"/>
       <x:c r="I96" s="14"/>
-      <x:c r="J96" s="14"/>
-      <x:c r="K96" s="14"/>
     </x:row>
     <x:row r="97" ht="23" customHeight="1">
       <x:c r="A97" s="14"/>
@@ -1620,8 +1424,6 @@
       <x:c r="G97" s="14"/>
       <x:c r="H97" s="14"/>
       <x:c r="I97" s="14"/>
-      <x:c r="J97" s="14"/>
-      <x:c r="K97" s="14"/>
     </x:row>
     <x:row r="98" ht="23" customHeight="1">
       <x:c r="A98" s="14"/>
@@ -1633,8 +1435,6 @@
       <x:c r="G98" s="14"/>
       <x:c r="H98" s="14"/>
       <x:c r="I98" s="14"/>
-      <x:c r="J98" s="14"/>
-      <x:c r="K98" s="14"/>
     </x:row>
     <x:row r="99" ht="23" customHeight="1">
       <x:c r="A99" s="14"/>
@@ -1646,8 +1446,6 @@
       <x:c r="G99" s="14"/>
       <x:c r="H99" s="14"/>
       <x:c r="I99" s="14"/>
-      <x:c r="J99" s="14"/>
-      <x:c r="K99" s="14"/>
     </x:row>
     <x:row r="100" ht="23" customHeight="1">
       <x:c r="A100" s="14"/>
@@ -1659,8 +1457,6 @@
       <x:c r="G100" s="14"/>
       <x:c r="H100" s="14"/>
       <x:c r="I100" s="14"/>
-      <x:c r="J100" s="14"/>
-      <x:c r="K100" s="14"/>
     </x:row>
     <x:row r="101" ht="23" customHeight="1">
       <x:c r="A101" s="14"/>
@@ -1672,8 +1468,6 @@
       <x:c r="G101" s="14"/>
       <x:c r="H101" s="14"/>
       <x:c r="I101" s="14"/>
-      <x:c r="J101" s="14"/>
-      <x:c r="K101" s="14"/>
     </x:row>
     <x:row r="102" ht="23" customHeight="1">
       <x:c r="A102" s="14"/>
@@ -1685,8 +1479,6 @@
       <x:c r="G102" s="14"/>
       <x:c r="H102" s="14"/>
       <x:c r="I102" s="14"/>
-      <x:c r="J102" s="14"/>
-      <x:c r="K102" s="14"/>
     </x:row>
     <x:row r="103" ht="23" customHeight="1">
       <x:c r="A103" s="14"/>
@@ -1698,8 +1490,6 @@
       <x:c r="G103" s="14"/>
       <x:c r="H103" s="14"/>
       <x:c r="I103" s="14"/>
-      <x:c r="J103" s="14"/>
-      <x:c r="K103" s="14"/>
     </x:row>
     <x:row r="104" ht="23" customHeight="1">
       <x:c r="A104" s="14"/>
@@ -1711,8 +1501,6 @@
       <x:c r="G104" s="14"/>
       <x:c r="H104" s="14"/>
       <x:c r="I104" s="14"/>
-      <x:c r="J104" s="14"/>
-      <x:c r="K104" s="14"/>
     </x:row>
     <x:row r="105" ht="23" customHeight="1">
       <x:c r="A105" s="14"/>
@@ -1724,8 +1512,6 @@
       <x:c r="G105" s="14"/>
       <x:c r="H105" s="14"/>
       <x:c r="I105" s="14"/>
-      <x:c r="J105" s="14"/>
-      <x:c r="K105" s="14"/>
     </x:row>
     <x:row r="106" ht="23" customHeight="1">
       <x:c r="A106" s="14"/>
@@ -1737,8 +1523,6 @@
       <x:c r="G106" s="14"/>
       <x:c r="H106" s="14"/>
       <x:c r="I106" s="14"/>
-      <x:c r="J106" s="14"/>
-      <x:c r="K106" s="14"/>
     </x:row>
     <x:row r="107" ht="23" customHeight="1">
       <x:c r="A107" s="14"/>
@@ -1750,8 +1534,6 @@
       <x:c r="G107" s="14"/>
       <x:c r="H107" s="14"/>
       <x:c r="I107" s="14"/>
-      <x:c r="J107" s="14"/>
-      <x:c r="K107" s="14"/>
     </x:row>
     <x:row r="108" ht="23" customHeight="1">
       <x:c r="A108" s="14"/>
@@ -1763,8 +1545,6 @@
       <x:c r="G108" s="14"/>
       <x:c r="H108" s="14"/>
       <x:c r="I108" s="14"/>
-      <x:c r="J108" s="14"/>
-      <x:c r="K108" s="14"/>
     </x:row>
     <x:row r="109" ht="23" customHeight="1">
       <x:c r="A109" s="14"/>
@@ -1776,8 +1556,6 @@
       <x:c r="G109" s="14"/>
       <x:c r="H109" s="14"/>
       <x:c r="I109" s="14"/>
-      <x:c r="J109" s="14"/>
-      <x:c r="K109" s="14"/>
     </x:row>
     <x:row r="110" ht="23" customHeight="1">
       <x:c r="A110" s="14"/>
@@ -1789,8 +1567,6 @@
       <x:c r="G110" s="14"/>
       <x:c r="H110" s="14"/>
       <x:c r="I110" s="14"/>
-      <x:c r="J110" s="14"/>
-      <x:c r="K110" s="14"/>
     </x:row>
     <x:row r="111" ht="23" customHeight="1">
       <x:c r="A111" s="14"/>
@@ -1802,8 +1578,6 @@
       <x:c r="G111" s="14"/>
       <x:c r="H111" s="14"/>
       <x:c r="I111" s="14"/>
-      <x:c r="J111" s="14"/>
-      <x:c r="K111" s="14"/>
     </x:row>
     <x:row r="112" ht="23" customHeight="1">
       <x:c r="A112" s="14"/>
@@ -1815,8 +1589,6 @@
       <x:c r="G112" s="14"/>
       <x:c r="H112" s="14"/>
       <x:c r="I112" s="14"/>
-      <x:c r="J112" s="14"/>
-      <x:c r="K112" s="14"/>
     </x:row>
     <x:row r="113" ht="23" customHeight="1">
       <x:c r="A113" s="14"/>
@@ -1828,8 +1600,6 @@
       <x:c r="G113" s="14"/>
       <x:c r="H113" s="14"/>
       <x:c r="I113" s="14"/>
-      <x:c r="J113" s="14"/>
-      <x:c r="K113" s="14"/>
     </x:row>
     <x:row r="114" ht="23" customHeight="1">
       <x:c r="A114" s="14"/>
@@ -1841,8 +1611,6 @@
       <x:c r="G114" s="14"/>
       <x:c r="H114" s="14"/>
       <x:c r="I114" s="14"/>
-      <x:c r="J114" s="14"/>
-      <x:c r="K114" s="14"/>
     </x:row>
     <x:row r="115" ht="23" customHeight="1">
       <x:c r="A115" s="14"/>
@@ -1854,8 +1622,6 @@
       <x:c r="G115" s="14"/>
       <x:c r="H115" s="14"/>
       <x:c r="I115" s="14"/>
-      <x:c r="J115" s="14"/>
-      <x:c r="K115" s="14"/>
     </x:row>
     <x:row r="116" ht="23" customHeight="1">
       <x:c r="A116" s="14"/>
@@ -1867,8 +1633,6 @@
       <x:c r="G116" s="14"/>
       <x:c r="H116" s="14"/>
       <x:c r="I116" s="14"/>
-      <x:c r="J116" s="14"/>
-      <x:c r="K116" s="14"/>
     </x:row>
     <x:row r="117" ht="23" customHeight="1">
       <x:c r="A117" s="14"/>
@@ -1880,8 +1644,6 @@
       <x:c r="G117" s="14"/>
       <x:c r="H117" s="14"/>
       <x:c r="I117" s="14"/>
-      <x:c r="J117" s="14"/>
-      <x:c r="K117" s="14"/>
     </x:row>
     <x:row r="118" ht="23" customHeight="1">
       <x:c r="A118" s="14"/>
@@ -1893,8 +1655,6 @@
       <x:c r="G118" s="14"/>
       <x:c r="H118" s="14"/>
       <x:c r="I118" s="14"/>
-      <x:c r="J118" s="14"/>
-      <x:c r="K118" s="14"/>
     </x:row>
     <x:row r="119" ht="23" customHeight="1">
       <x:c r="A119" s="14"/>
@@ -1906,8 +1666,6 @@
       <x:c r="G119" s="14"/>
       <x:c r="H119" s="14"/>
       <x:c r="I119" s="14"/>
-      <x:c r="J119" s="14"/>
-      <x:c r="K119" s="14"/>
     </x:row>
     <x:row r="120" ht="23" customHeight="1">
       <x:c r="A120" s="14"/>
@@ -1919,8 +1677,6 @@
       <x:c r="G120" s="14"/>
       <x:c r="H120" s="14"/>
       <x:c r="I120" s="14"/>
-      <x:c r="J120" s="14"/>
-      <x:c r="K120" s="14"/>
     </x:row>
     <x:row r="121" ht="23" customHeight="1">
       <x:c r="A121" s="14"/>
@@ -1932,8 +1688,6 @@
       <x:c r="G121" s="14"/>
       <x:c r="H121" s="14"/>
       <x:c r="I121" s="14"/>
-      <x:c r="J121" s="14"/>
-      <x:c r="K121" s="14"/>
     </x:row>
     <x:row r="122" ht="23" customHeight="1">
       <x:c r="A122" s="14"/>
@@ -1945,8 +1699,6 @@
       <x:c r="G122" s="14"/>
       <x:c r="H122" s="14"/>
       <x:c r="I122" s="14"/>
-      <x:c r="J122" s="14"/>
-      <x:c r="K122" s="14"/>
     </x:row>
     <x:row r="123" ht="23" customHeight="1">
       <x:c r="A123" s="14"/>
@@ -1958,8 +1710,6 @@
       <x:c r="G123" s="14"/>
       <x:c r="H123" s="14"/>
       <x:c r="I123" s="14"/>
-      <x:c r="J123" s="14"/>
-      <x:c r="K123" s="14"/>
     </x:row>
     <x:row r="124" ht="23" customHeight="1">
       <x:c r="A124" s="14"/>
@@ -1971,8 +1721,6 @@
       <x:c r="G124" s="14"/>
       <x:c r="H124" s="14"/>
       <x:c r="I124" s="14"/>
-      <x:c r="J124" s="14"/>
-      <x:c r="K124" s="14"/>
     </x:row>
     <x:row r="125" ht="23" customHeight="1">
       <x:c r="A125" s="14"/>
@@ -1984,8 +1732,6 @@
       <x:c r="G125" s="14"/>
       <x:c r="H125" s="14"/>
       <x:c r="I125" s="14"/>
-      <x:c r="J125" s="14"/>
-      <x:c r="K125" s="14"/>
     </x:row>
     <x:row r="126" ht="23" customHeight="1">
       <x:c r="A126" s="14"/>
@@ -1997,8 +1743,6 @@
       <x:c r="G126" s="14"/>
       <x:c r="H126" s="14"/>
       <x:c r="I126" s="14"/>
-      <x:c r="J126" s="14"/>
-      <x:c r="K126" s="14"/>
     </x:row>
     <x:row r="127" ht="23" customHeight="1">
       <x:c r="A127" s="14"/>
@@ -2010,8 +1754,6 @@
       <x:c r="G127" s="14"/>
       <x:c r="H127" s="14"/>
       <x:c r="I127" s="14"/>
-      <x:c r="J127" s="14"/>
-      <x:c r="K127" s="14"/>
     </x:row>
     <x:row r="128" ht="23" customHeight="1">
       <x:c r="A128" s="14"/>
@@ -2023,8 +1765,6 @@
       <x:c r="G128" s="14"/>
       <x:c r="H128" s="14"/>
       <x:c r="I128" s="14"/>
-      <x:c r="J128" s="14"/>
-      <x:c r="K128" s="14"/>
     </x:row>
     <x:row r="129" ht="23" customHeight="1">
       <x:c r="A129" s="14"/>
@@ -2036,8 +1776,6 @@
       <x:c r="G129" s="14"/>
       <x:c r="H129" s="14"/>
       <x:c r="I129" s="14"/>
-      <x:c r="J129" s="14"/>
-      <x:c r="K129" s="14"/>
     </x:row>
     <x:row r="130" ht="23" customHeight="1">
       <x:c r="A130" s="14"/>
@@ -2049,8 +1787,6 @@
       <x:c r="G130" s="14"/>
       <x:c r="H130" s="14"/>
       <x:c r="I130" s="14"/>
-      <x:c r="J130" s="14"/>
-      <x:c r="K130" s="14"/>
     </x:row>
     <x:row r="131" ht="23" customHeight="1">
       <x:c r="A131" s="14"/>
@@ -2062,8 +1798,6 @@
       <x:c r="G131" s="14"/>
       <x:c r="H131" s="14"/>
       <x:c r="I131" s="14"/>
-      <x:c r="J131" s="14"/>
-      <x:c r="K131" s="14"/>
     </x:row>
     <x:row r="132" ht="23" customHeight="1">
       <x:c r="A132" s="14"/>
@@ -2075,8 +1809,6 @@
       <x:c r="G132" s="14"/>
       <x:c r="H132" s="14"/>
       <x:c r="I132" s="14"/>
-      <x:c r="J132" s="14"/>
-      <x:c r="K132" s="14"/>
     </x:row>
     <x:row r="133" ht="23" customHeight="1">
       <x:c r="A133" s="14"/>
@@ -2088,8 +1820,6 @@
       <x:c r="G133" s="14"/>
       <x:c r="H133" s="14"/>
       <x:c r="I133" s="14"/>
-      <x:c r="J133" s="14"/>
-      <x:c r="K133" s="14"/>
     </x:row>
     <x:row r="134" ht="23" customHeight="1">
       <x:c r="A134" s="14"/>
@@ -2101,8 +1831,6 @@
       <x:c r="G134" s="14"/>
       <x:c r="H134" s="14"/>
       <x:c r="I134" s="14"/>
-      <x:c r="J134" s="14"/>
-      <x:c r="K134" s="14"/>
     </x:row>
     <x:row r="135" ht="23" customHeight="1">
       <x:c r="A135" s="14"/>
@@ -2114,8 +1842,6 @@
       <x:c r="G135" s="14"/>
       <x:c r="H135" s="14"/>
       <x:c r="I135" s="14"/>
-      <x:c r="J135" s="14"/>
-      <x:c r="K135" s="14"/>
     </x:row>
     <x:row r="136" ht="23" customHeight="1">
       <x:c r="A136" s="14"/>
@@ -2127,8 +1853,6 @@
       <x:c r="G136" s="14"/>
       <x:c r="H136" s="14"/>
       <x:c r="I136" s="14"/>
-      <x:c r="J136" s="14"/>
-      <x:c r="K136" s="14"/>
     </x:row>
     <x:row r="137" ht="23" customHeight="1">
       <x:c r="A137" s="14"/>
@@ -2140,8 +1864,6 @@
       <x:c r="G137" s="14"/>
       <x:c r="H137" s="14"/>
       <x:c r="I137" s="14"/>
-      <x:c r="J137" s="14"/>
-      <x:c r="K137" s="14"/>
     </x:row>
     <x:row r="138" ht="23" customHeight="1">
       <x:c r="A138" s="14"/>
@@ -2153,8 +1875,6 @@
       <x:c r="G138" s="14"/>
       <x:c r="H138" s="14"/>
       <x:c r="I138" s="14"/>
-      <x:c r="J138" s="14"/>
-      <x:c r="K138" s="14"/>
     </x:row>
     <x:row r="139" ht="23" customHeight="1">
       <x:c r="A139" s="14"/>
@@ -2166,8 +1886,6 @@
       <x:c r="G139" s="14"/>
       <x:c r="H139" s="14"/>
       <x:c r="I139" s="14"/>
-      <x:c r="J139" s="14"/>
-      <x:c r="K139" s="14"/>
     </x:row>
     <x:row r="140" ht="23" customHeight="1">
       <x:c r="A140" s="14"/>
@@ -2179,8 +1897,6 @@
       <x:c r="G140" s="14"/>
       <x:c r="H140" s="14"/>
       <x:c r="I140" s="14"/>
-      <x:c r="J140" s="14"/>
-      <x:c r="K140" s="14"/>
     </x:row>
     <x:row r="141" ht="23" customHeight="1">
       <x:c r="A141" s="14"/>
@@ -2192,8 +1908,6 @@
       <x:c r="G141" s="14"/>
       <x:c r="H141" s="14"/>
       <x:c r="I141" s="14"/>
-      <x:c r="J141" s="14"/>
-      <x:c r="K141" s="14"/>
     </x:row>
     <x:row r="142" ht="23" customHeight="1">
       <x:c r="A142" s="14"/>
@@ -2205,8 +1919,6 @@
       <x:c r="G142" s="14"/>
       <x:c r="H142" s="14"/>
       <x:c r="I142" s="14"/>
-      <x:c r="J142" s="14"/>
-      <x:c r="K142" s="14"/>
     </x:row>
     <x:row r="143" ht="23" customHeight="1">
       <x:c r="A143" s="14"/>
@@ -2218,8 +1930,6 @@
       <x:c r="G143" s="14"/>
       <x:c r="H143" s="14"/>
       <x:c r="I143" s="14"/>
-      <x:c r="J143" s="14"/>
-      <x:c r="K143" s="14"/>
     </x:row>
     <x:row r="144" ht="23" customHeight="1">
       <x:c r="A144" s="14"/>
@@ -2231,8 +1941,6 @@
       <x:c r="G144" s="14"/>
       <x:c r="H144" s="14"/>
       <x:c r="I144" s="14"/>
-      <x:c r="J144" s="14"/>
-      <x:c r="K144" s="14"/>
     </x:row>
     <x:row r="145" ht="23" customHeight="1">
       <x:c r="A145" s="14"/>
@@ -2244,8 +1952,6 @@
       <x:c r="G145" s="14"/>
       <x:c r="H145" s="14"/>
       <x:c r="I145" s="14"/>
-      <x:c r="J145" s="14"/>
-      <x:c r="K145" s="14"/>
     </x:row>
     <x:row r="146" ht="23" customHeight="1">
       <x:c r="A146" s="14"/>
@@ -2257,8 +1963,6 @@
       <x:c r="G146" s="14"/>
       <x:c r="H146" s="14"/>
       <x:c r="I146" s="14"/>
-      <x:c r="J146" s="14"/>
-      <x:c r="K146" s="14"/>
     </x:row>
     <x:row r="147" ht="23" customHeight="1">
       <x:c r="A147" s="14"/>
@@ -2270,8 +1974,6 @@
       <x:c r="G147" s="14"/>
       <x:c r="H147" s="14"/>
       <x:c r="I147" s="14"/>
-      <x:c r="J147" s="14"/>
-      <x:c r="K147" s="14"/>
     </x:row>
     <x:row r="148" ht="23" customHeight="1">
       <x:c r="A148" s="14"/>
@@ -2283,8 +1985,6 @@
       <x:c r="G148" s="14"/>
       <x:c r="H148" s="14"/>
       <x:c r="I148" s="14"/>
-      <x:c r="J148" s="14"/>
-      <x:c r="K148" s="14"/>
     </x:row>
     <x:row r="149" ht="23" customHeight="1">
       <x:c r="A149" s="14"/>
@@ -2296,8 +1996,6 @@
       <x:c r="G149" s="14"/>
       <x:c r="H149" s="14"/>
       <x:c r="I149" s="14"/>
-      <x:c r="J149" s="14"/>
-      <x:c r="K149" s="14"/>
     </x:row>
     <x:row r="150" ht="23" customHeight="1">
       <x:c r="A150" s="14"/>
@@ -2309,8 +2007,6 @@
       <x:c r="G150" s="14"/>
       <x:c r="H150" s="14"/>
       <x:c r="I150" s="14"/>
-      <x:c r="J150" s="14"/>
-      <x:c r="K150" s="14"/>
     </x:row>
     <x:row r="151" ht="23" customHeight="1">
       <x:c r="A151" s="14"/>
@@ -2322,8 +2018,6 @@
       <x:c r="G151" s="14"/>
       <x:c r="H151" s="14"/>
       <x:c r="I151" s="14"/>
-      <x:c r="J151" s="14"/>
-      <x:c r="K151" s="14"/>
     </x:row>
     <x:row r="152" ht="23" customHeight="1">
       <x:c r="A152" s="14"/>
@@ -2335,8 +2029,6 @@
       <x:c r="G152" s="14"/>
       <x:c r="H152" s="14"/>
       <x:c r="I152" s="14"/>
-      <x:c r="J152" s="14"/>
-      <x:c r="K152" s="14"/>
     </x:row>
     <x:row r="153" ht="23" customHeight="1">
       <x:c r="A153" s="14"/>
@@ -2348,8 +2040,6 @@
       <x:c r="G153" s="14"/>
       <x:c r="H153" s="14"/>
       <x:c r="I153" s="14"/>
-      <x:c r="J153" s="14"/>
-      <x:c r="K153" s="14"/>
     </x:row>
     <x:row r="154" ht="23" customHeight="1">
       <x:c r="A154" s="14"/>
@@ -2361,8 +2051,6 @@
       <x:c r="G154" s="14"/>
       <x:c r="H154" s="14"/>
       <x:c r="I154" s="14"/>
-      <x:c r="J154" s="14"/>
-      <x:c r="K154" s="14"/>
     </x:row>
     <x:row r="155" ht="23" customHeight="1">
       <x:c r="A155" s="14"/>
@@ -2374,8 +2062,6 @@
       <x:c r="G155" s="14"/>
       <x:c r="H155" s="14"/>
       <x:c r="I155" s="14"/>
-      <x:c r="J155" s="14"/>
-      <x:c r="K155" s="14"/>
     </x:row>
     <x:row r="156" ht="23" customHeight="1">
       <x:c r="A156" s="14"/>
@@ -2387,8 +2073,6 @@
       <x:c r="G156" s="14"/>
       <x:c r="H156" s="14"/>
       <x:c r="I156" s="14"/>
-      <x:c r="J156" s="14"/>
-      <x:c r="K156" s="14"/>
     </x:row>
     <x:row r="157" ht="23" customHeight="1">
       <x:c r="A157" s="14"/>
@@ -2400,8 +2084,6 @@
       <x:c r="G157" s="14"/>
       <x:c r="H157" s="14"/>
       <x:c r="I157" s="14"/>
-      <x:c r="J157" s="14"/>
-      <x:c r="K157" s="14"/>
     </x:row>
     <x:row r="158" ht="23" customHeight="1">
       <x:c r="A158" s="14"/>
@@ -2413,8 +2095,6 @@
       <x:c r="G158" s="14"/>
       <x:c r="H158" s="14"/>
       <x:c r="I158" s="14"/>
-      <x:c r="J158" s="14"/>
-      <x:c r="K158" s="14"/>
     </x:row>
     <x:row r="159" ht="23" customHeight="1">
       <x:c r="A159" s="14"/>
@@ -2426,8 +2106,6 @@
       <x:c r="G159" s="14"/>
       <x:c r="H159" s="14"/>
       <x:c r="I159" s="14"/>
-      <x:c r="J159" s="14"/>
-      <x:c r="K159" s="14"/>
     </x:row>
     <x:row r="160" ht="23" customHeight="1">
       <x:c r="A160" s="14"/>
@@ -2439,8 +2117,6 @@
       <x:c r="G160" s="14"/>
       <x:c r="H160" s="14"/>
       <x:c r="I160" s="14"/>
-      <x:c r="J160" s="14"/>
-      <x:c r="K160" s="14"/>
     </x:row>
     <x:row r="161" ht="23" customHeight="1">
       <x:c r="A161" s="14"/>
@@ -2452,8 +2128,6 @@
       <x:c r="G161" s="14"/>
       <x:c r="H161" s="14"/>
       <x:c r="I161" s="14"/>
-      <x:c r="J161" s="14"/>
-      <x:c r="K161" s="14"/>
     </x:row>
     <x:row r="162" ht="23" customHeight="1">
       <x:c r="A162" s="14"/>
@@ -2465,8 +2139,6 @@
       <x:c r="G162" s="14"/>
       <x:c r="H162" s="14"/>
       <x:c r="I162" s="14"/>
-      <x:c r="J162" s="14"/>
-      <x:c r="K162" s="14"/>
     </x:row>
     <x:row r="163" ht="23" customHeight="1">
       <x:c r="A163" s="14"/>
@@ -2478,8 +2150,6 @@
       <x:c r="G163" s="14"/>
       <x:c r="H163" s="14"/>
       <x:c r="I163" s="14"/>
-      <x:c r="J163" s="14"/>
-      <x:c r="K163" s="14"/>
     </x:row>
     <x:row r="164" ht="23" customHeight="1">
       <x:c r="A164" s="14"/>
@@ -2491,8 +2161,6 @@
       <x:c r="G164" s="14"/>
       <x:c r="H164" s="14"/>
       <x:c r="I164" s="14"/>
-      <x:c r="J164" s="14"/>
-      <x:c r="K164" s="14"/>
     </x:row>
     <x:row r="165" ht="23" customHeight="1">
       <x:c r="A165" s="14"/>
@@ -2504,8 +2172,6 @@
       <x:c r="G165" s="14"/>
       <x:c r="H165" s="14"/>
       <x:c r="I165" s="14"/>
-      <x:c r="J165" s="14"/>
-      <x:c r="K165" s="14"/>
     </x:row>
     <x:row r="166" ht="23" customHeight="1">
       <x:c r="A166" s="14"/>
@@ -2517,8 +2183,6 @@
       <x:c r="G166" s="14"/>
       <x:c r="H166" s="14"/>
       <x:c r="I166" s="14"/>
-      <x:c r="J166" s="14"/>
-      <x:c r="K166" s="14"/>
     </x:row>
     <x:row r="167" ht="23" customHeight="1">
       <x:c r="A167" s="14"/>
@@ -2530,8 +2194,6 @@
       <x:c r="G167" s="14"/>
       <x:c r="H167" s="14"/>
       <x:c r="I167" s="14"/>
-      <x:c r="J167" s="14"/>
-      <x:c r="K167" s="14"/>
     </x:row>
     <x:row r="168" ht="23" customHeight="1">
       <x:c r="A168" s="14"/>
@@ -2543,8 +2205,6 @@
       <x:c r="G168" s="14"/>
       <x:c r="H168" s="14"/>
       <x:c r="I168" s="14"/>
-      <x:c r="J168" s="14"/>
-      <x:c r="K168" s="14"/>
     </x:row>
     <x:row r="169" ht="23" customHeight="1">
       <x:c r="A169" s="14"/>
@@ -2556,8 +2216,6 @@
       <x:c r="G169" s="14"/>
       <x:c r="H169" s="14"/>
       <x:c r="I169" s="14"/>
-      <x:c r="J169" s="14"/>
-      <x:c r="K169" s="14"/>
     </x:row>
     <x:row r="170" ht="23" customHeight="1">
       <x:c r="A170" s="14"/>
@@ -2569,8 +2227,6 @@
       <x:c r="G170" s="14"/>
       <x:c r="H170" s="14"/>
       <x:c r="I170" s="14"/>
-      <x:c r="J170" s="14"/>
-      <x:c r="K170" s="14"/>
     </x:row>
     <x:row r="171" ht="23" customHeight="1">
       <x:c r="A171" s="14"/>
@@ -2582,8 +2238,6 @@
       <x:c r="G171" s="14"/>
       <x:c r="H171" s="14"/>
       <x:c r="I171" s="14"/>
-      <x:c r="J171" s="14"/>
-      <x:c r="K171" s="14"/>
     </x:row>
     <x:row r="172" ht="23" customHeight="1">
       <x:c r="A172" s="14"/>
@@ -2595,8 +2249,6 @@
       <x:c r="G172" s="14"/>
       <x:c r="H172" s="14"/>
       <x:c r="I172" s="14"/>
-      <x:c r="J172" s="14"/>
-      <x:c r="K172" s="14"/>
     </x:row>
     <x:row r="173" ht="23" customHeight="1">
       <x:c r="A173" s="14"/>
@@ -2608,8 +2260,6 @@
       <x:c r="G173" s="14"/>
       <x:c r="H173" s="14"/>
       <x:c r="I173" s="14"/>
-      <x:c r="J173" s="14"/>
-      <x:c r="K173" s="14"/>
     </x:row>
     <x:row r="174" ht="23" customHeight="1">
       <x:c r="A174" s="14"/>
@@ -2621,8 +2271,6 @@
       <x:c r="G174" s="14"/>
       <x:c r="H174" s="14"/>
       <x:c r="I174" s="14"/>
-      <x:c r="J174" s="14"/>
-      <x:c r="K174" s="14"/>
     </x:row>
     <x:row r="175" ht="23" customHeight="1">
       <x:c r="A175" s="14"/>
@@ -2634,8 +2282,6 @@
       <x:c r="G175" s="14"/>
       <x:c r="H175" s="14"/>
       <x:c r="I175" s="14"/>
-      <x:c r="J175" s="14"/>
-      <x:c r="K175" s="14"/>
     </x:row>
     <x:row r="176" ht="23" customHeight="1">
       <x:c r="A176" s="14"/>
@@ -2647,8 +2293,6 @@
       <x:c r="G176" s="14"/>
       <x:c r="H176" s="14"/>
       <x:c r="I176" s="14"/>
-      <x:c r="J176" s="14"/>
-      <x:c r="K176" s="14"/>
     </x:row>
     <x:row r="177" ht="23" customHeight="1">
       <x:c r="A177" s="14"/>
@@ -2660,8 +2304,6 @@
       <x:c r="G177" s="14"/>
       <x:c r="H177" s="14"/>
       <x:c r="I177" s="14"/>
-      <x:c r="J177" s="14"/>
-      <x:c r="K177" s="14"/>
     </x:row>
     <x:row r="178" ht="23" customHeight="1">
       <x:c r="A178" s="14"/>
@@ -2673,8 +2315,6 @@
       <x:c r="G178" s="14"/>
       <x:c r="H178" s="14"/>
       <x:c r="I178" s="14"/>
-      <x:c r="J178" s="14"/>
-      <x:c r="K178" s="14"/>
     </x:row>
     <x:row r="179" ht="23" customHeight="1">
       <x:c r="A179" s="14"/>
@@ -2686,8 +2326,6 @@
       <x:c r="G179" s="14"/>
       <x:c r="H179" s="14"/>
       <x:c r="I179" s="14"/>
-      <x:c r="J179" s="14"/>
-      <x:c r="K179" s="14"/>
     </x:row>
     <x:row r="180" ht="23" customHeight="1">
       <x:c r="A180" s="14"/>
@@ -2699,8 +2337,6 @@
       <x:c r="G180" s="14"/>
       <x:c r="H180" s="14"/>
       <x:c r="I180" s="14"/>
-      <x:c r="J180" s="14"/>
-      <x:c r="K180" s="14"/>
     </x:row>
     <x:row r="181" ht="23" customHeight="1">
       <x:c r="A181" s="14"/>
@@ -2712,8 +2348,6 @@
       <x:c r="G181" s="14"/>
       <x:c r="H181" s="14"/>
       <x:c r="I181" s="14"/>
-      <x:c r="J181" s="14"/>
-      <x:c r="K181" s="14"/>
     </x:row>
     <x:row r="182" ht="23" customHeight="1">
       <x:c r="A182" s="14"/>
@@ -2725,8 +2359,6 @@
       <x:c r="G182" s="14"/>
       <x:c r="H182" s="14"/>
       <x:c r="I182" s="14"/>
-      <x:c r="J182" s="14"/>
-      <x:c r="K182" s="14"/>
     </x:row>
     <x:row r="183" ht="23" customHeight="1">
       <x:c r="A183" s="14"/>
@@ -2738,8 +2370,6 @@
       <x:c r="G183" s="14"/>
       <x:c r="H183" s="14"/>
       <x:c r="I183" s="14"/>
-      <x:c r="J183" s="14"/>
-      <x:c r="K183" s="14"/>
     </x:row>
     <x:row r="184" ht="23" customHeight="1">
       <x:c r="A184" s="14"/>
@@ -2751,8 +2381,6 @@
       <x:c r="G184" s="14"/>
       <x:c r="H184" s="14"/>
       <x:c r="I184" s="14"/>
-      <x:c r="J184" s="14"/>
-      <x:c r="K184" s="14"/>
     </x:row>
     <x:row r="185" ht="23" customHeight="1">
       <x:c r="A185" s="14"/>
@@ -2764,8 +2392,6 @@
       <x:c r="G185" s="14"/>
       <x:c r="H185" s="14"/>
       <x:c r="I185" s="14"/>
-      <x:c r="J185" s="14"/>
-      <x:c r="K185" s="14"/>
     </x:row>
     <x:row r="186" ht="23" customHeight="1">
       <x:c r="A186" s="14"/>
@@ -2777,8 +2403,6 @@
       <x:c r="G186" s="14"/>
       <x:c r="H186" s="14"/>
       <x:c r="I186" s="14"/>
-      <x:c r="J186" s="14"/>
-      <x:c r="K186" s="14"/>
     </x:row>
     <x:row r="187" ht="23" customHeight="1">
       <x:c r="A187" s="14"/>
@@ -2790,8 +2414,6 @@
       <x:c r="G187" s="14"/>
       <x:c r="H187" s="14"/>
       <x:c r="I187" s="14"/>
-      <x:c r="J187" s="14"/>
-      <x:c r="K187" s="14"/>
     </x:row>
     <x:row r="188" ht="23" customHeight="1">
       <x:c r="A188" s="14"/>
@@ -2803,8 +2425,6 @@
       <x:c r="G188" s="14"/>
       <x:c r="H188" s="14"/>
       <x:c r="I188" s="14"/>
-      <x:c r="J188" s="14"/>
-      <x:c r="K188" s="14"/>
     </x:row>
     <x:row r="189" ht="23" customHeight="1">
       <x:c r="A189" s="14"/>
@@ -2816,8 +2436,6 @@
       <x:c r="G189" s="14"/>
       <x:c r="H189" s="14"/>
       <x:c r="I189" s="14"/>
-      <x:c r="J189" s="14"/>
-      <x:c r="K189" s="14"/>
     </x:row>
     <x:row r="190" ht="23" customHeight="1">
       <x:c r="A190" s="14"/>
@@ -2829,8 +2447,6 @@
       <x:c r="G190" s="14"/>
       <x:c r="H190" s="14"/>
       <x:c r="I190" s="14"/>
-      <x:c r="J190" s="14"/>
-      <x:c r="K190" s="14"/>
     </x:row>
     <x:row r="191" ht="23" customHeight="1">
       <x:c r="A191" s="14"/>
@@ -2842,8 +2458,6 @@
       <x:c r="G191" s="14"/>
       <x:c r="H191" s="14"/>
       <x:c r="I191" s="14"/>
-      <x:c r="J191" s="14"/>
-      <x:c r="K191" s="14"/>
     </x:row>
     <x:row r="192" ht="23" customHeight="1">
       <x:c r="A192" s="14"/>
@@ -2855,8 +2469,6 @@
       <x:c r="G192" s="14"/>
       <x:c r="H192" s="14"/>
       <x:c r="I192" s="14"/>
-      <x:c r="J192" s="14"/>
-      <x:c r="K192" s="14"/>
     </x:row>
     <x:row r="193" ht="23" customHeight="1">
       <x:c r="A193" s="14"/>
@@ -2868,8 +2480,6 @@
       <x:c r="G193" s="14"/>
       <x:c r="H193" s="14"/>
       <x:c r="I193" s="14"/>
-      <x:c r="J193" s="14"/>
-      <x:c r="K193" s="14"/>
     </x:row>
     <x:row r="194" ht="23" customHeight="1">
       <x:c r="A194" s="14"/>
@@ -2881,8 +2491,6 @@
       <x:c r="G194" s="14"/>
       <x:c r="H194" s="14"/>
       <x:c r="I194" s="14"/>
-      <x:c r="J194" s="14"/>
-      <x:c r="K194" s="14"/>
     </x:row>
     <x:row r="195" ht="23" customHeight="1">
       <x:c r="A195" s="14"/>
@@ -2894,8 +2502,6 @@
       <x:c r="G195" s="14"/>
       <x:c r="H195" s="14"/>
       <x:c r="I195" s="14"/>
-      <x:c r="J195" s="14"/>
-      <x:c r="K195" s="14"/>
     </x:row>
     <x:row r="196" ht="23" customHeight="1">
       <x:c r="A196" s="14"/>
@@ -2907,8 +2513,6 @@
       <x:c r="G196" s="14"/>
       <x:c r="H196" s="14"/>
       <x:c r="I196" s="14"/>
-      <x:c r="J196" s="14"/>
-      <x:c r="K196" s="14"/>
     </x:row>
     <x:row r="197" ht="23" customHeight="1">
       <x:c r="A197" s="14"/>
@@ -2920,8 +2524,6 @@
       <x:c r="G197" s="14"/>
       <x:c r="H197" s="14"/>
       <x:c r="I197" s="14"/>
-      <x:c r="J197" s="14"/>
-      <x:c r="K197" s="14"/>
     </x:row>
     <x:row r="198" ht="23" customHeight="1">
       <x:c r="A198" s="14"/>
@@ -2933,8 +2535,6 @@
       <x:c r="G198" s="14"/>
       <x:c r="H198" s="14"/>
       <x:c r="I198" s="14"/>
-      <x:c r="J198" s="14"/>
-      <x:c r="K198" s="14"/>
     </x:row>
     <x:row r="199" ht="23" customHeight="1">
       <x:c r="A199" s="14"/>
@@ -2946,8 +2546,6 @@
       <x:c r="G199" s="14"/>
       <x:c r="H199" s="14"/>
       <x:c r="I199" s="14"/>
-      <x:c r="J199" s="14"/>
-      <x:c r="K199" s="14"/>
     </x:row>
     <x:row r="200" ht="23" customHeight="1">
       <x:c r="A200" s="14"/>
@@ -2959,8 +2557,6 @@
       <x:c r="G200" s="14"/>
       <x:c r="H200" s="14"/>
       <x:c r="I200" s="14"/>
-      <x:c r="J200" s="14"/>
-      <x:c r="K200" s="14"/>
     </x:row>
     <x:row r="201" ht="23" customHeight="1">
       <x:c r="A201" s="14"/>
@@ -2972,8 +2568,6 @@
       <x:c r="G201" s="14"/>
       <x:c r="H201" s="14"/>
       <x:c r="I201" s="14"/>
-      <x:c r="J201" s="14"/>
-      <x:c r="K201" s="14"/>
     </x:row>
     <x:row r="202" ht="23" customHeight="1">
       <x:c r="A202" s="14"/>
@@ -2985,8 +2579,6 @@
       <x:c r="G202" s="14"/>
       <x:c r="H202" s="14"/>
       <x:c r="I202" s="14"/>
-      <x:c r="J202" s="14"/>
-      <x:c r="K202" s="14"/>
     </x:row>
     <x:row r="203" ht="23" customHeight="1">
       <x:c r="A203" s="14"/>
@@ -2998,8 +2590,6 @@
       <x:c r="G203" s="14"/>
       <x:c r="H203" s="14"/>
       <x:c r="I203" s="14"/>
-      <x:c r="J203" s="14"/>
-      <x:c r="K203" s="14"/>
     </x:row>
     <x:row r="204" ht="23" customHeight="1">
       <x:c r="A204" s="14"/>
@@ -3011,8 +2601,6 @@
       <x:c r="G204" s="14"/>
       <x:c r="H204" s="14"/>
       <x:c r="I204" s="14"/>
-      <x:c r="J204" s="14"/>
-      <x:c r="K204" s="14"/>
     </x:row>
     <x:row r="205" ht="23" customHeight="1">
       <x:c r="A205" s="14"/>
@@ -3024,12 +2612,10 @@
       <x:c r="G205" s="14"/>
       <x:c r="H205" s="14"/>
       <x:c r="I205" s="14"/>
-      <x:c r="J205" s="14"/>
-      <x:c r="K205" s="14"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="J6:J205">
+    <x:dataValidation type="list" sqref="H6:H205">
       <x:formula1>"published,draft"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -3130,7 +2716,7 @@
         <x:v>Capacity / 名额</x:v>
       </x:c>
       <x:c r="B10" s="14" t="str">
-        <x:v>Enter a whole number from 1 to 1000. / 填写 1 至 1000 的整数。</x:v>
+        <x:v>Enter a whole number from 0 to 1000; 0 shows the session as full. / 填写 0 至 1000 的整数；0 表示该场次显示为已满。</x:v>
       </x:c>
       <x:c r="C10" s="14" t="str">
         <x:v>12</x:v>
@@ -3149,43 +2735,32 @@
     </x:row>
     <x:row r="12" ht="38" customHeight="1">
       <x:c r="A12" s="14" t="str">
-        <x:v>Descriptions (optional) / 活动介绍（可选）</x:v>
+        <x:v>Status / 状态</x:v>
       </x:c>
       <x:c r="B12" s="14" t="str">
-        <x:v>Both English and Chinese descriptions are optional; blank cells are generated from the session details. Max 2000 characters each. / 英文和中文介绍均可留空，留空后会根据场次信息自动生成；每项最多 2000 字符。</x:v>
+        <x:v>Choose published or draft. Blank defaults to draft. / 选择 published 或 draft；留空默认为草稿。</x:v>
       </x:c>
       <x:c r="C12" s="14" t="str">
-        <x:v>Friendly doubles session</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="38" customHeight="1">
+        <x:v>draft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="64" customHeight="1">
       <x:c r="A13" s="14" t="str">
-        <x:v>Status / 状态</x:v>
+        <x:v>Duplicate sessions / 重复场次</x:v>
       </x:c>
       <x:c r="B13" s="14" t="str">
-        <x:v>Choose published or draft. Blank defaults to draft. / 选择 published 或 draft；留空默认为草稿。</x:v>
-      </x:c>
-      <x:c r="C13" s="14" t="str">
-        <x:v>draft</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="64" customHeight="1">
+        <x:v>The same venue, date, start time and end time cannot already exist or appear twice in one import. Failed rows show their specific reasons. / 同一场地、日期、开始和结束时间不能与已有场次或本次文件中的其他场次重复。导入失败时会显示具体行和原因。</x:v>
+      </x:c>
+      <x:c r="C13" s="14" t="str"/>
+    </x:row>
+    <x:row r="14" ht="38" customHeight="1">
       <x:c r="A14" s="14" t="str">
-        <x:v>Duplicate sessions / 重复场次</x:v>
+        <x:v>Save as .xlsx / 保存为 .xlsx</x:v>
       </x:c>
       <x:c r="B14" s="14" t="str">
-        <x:v>The same venue, date, start time and end time cannot already exist or appear twice in one import. Failed rows show their specific reasons. / 同一场地、日期、开始和结束时间不能与已有场次或本次文件中的其他场次重复。导入失败时会显示具体行和原因。</x:v>
+        <x:v>Keep the first Sessions sheet and its column headers intact. / 保留第一个 Sessions 工作表和列标题。</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str"/>
-    </x:row>
-    <x:row r="15" ht="38" customHeight="1">
-      <x:c r="A15" s="14" t="str">
-        <x:v>Save as .xlsx / 保存为 .xlsx</x:v>
-      </x:c>
-      <x:c r="B15" s="14" t="str">
-        <x:v>Keep the first Sessions sheet and its column headers intact. / 保留第一个 Sessions 工作表和列标题。</x:v>
-      </x:c>
-      <x:c r="C15" s="14" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>